<commit_message>
Update village feed (24h lookback)
</commit_message>
<xml_diff>
--- a/data/google_news_dedup_10_0426_UTC_past2d.xlsx
+++ b/data/google_news_dedup_10_0426_UTC_past2d.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K101"/>
+  <dimension ref="A1:K84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,32 +480,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BV Logistics Companies</t>
+          <t>Brand Protest</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>("Dropit" OR "DHL" OR "UPS" OR "DPD" OR "Flight Logistics" OR "Fedex" OR "Amazon" OR "Royal Mail" OR "Parcelforce" OR "EVRI" ) AND ( "supply " OR  "delivery") AND -"postal vote"</t>
+          <t>("Gucci" OR "Ralph Lauren" OR "Dior" OR "Armani" OR "Louis Vuitton" OR "Burberry" OR "Prada" OR "Nike" OR "Canada Goose" OR "Hugo Boss" OR "Moncler" OR "Saint Laurent" OR "Loro Piana" OR "Lacoste" OR "Versace" OR "Jimmy Choo" OR "Michael Kors" OR "Missoni" OR "Kiton" OR "Aquazzura" OR "Tumi") AND ("protest" OR "animal rights" OR "fur free" OR "PETA" OR "activist") AND -BAFTA AND -"red carpet" AND -"awards" AND -"wears" AND -"dressed in"</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CEO Andy Jassy’s 2025 Letter to Shareholders - About Amazon</t>
+          <t>Morning Coffee: When executive assistants steal from bankers and buy handbags. The joy of being Apollo - eFinancialCareers</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>CEO Andy Jassy’s 2025 Letter to Shareholders - About Amazon</t>
+          <t>Morning Coffee: When executive assistants steal from bankers and buy handbags. The joy of being Apollo - eFinancialCareers</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 10:07:13 GMT</t>
+          <t>Fri, 10 Apr 2026 09:08:29 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxObWFDWFp0cEY5ZUFqd01nYmlLVWg0cjBreFFXaFMxZGFOV085T3RNVDdsRTlwcFpPb3E3MnkwbjNjVlRaWjVDNjAtSkUzZGtKSHpiVWJZc1BjVXNsdlR6TEdhd1hKTlM0aVJWUHNKUEppSlh2OHhwYjVFTVhyVC1oZ2RSNnJzVHV1UkRna09wcVBwdlFoSWkwdTBVQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTFBFNUt6YWtoQThmdzVRWGZiWnBpRkhOZUdZSUdzNkg0eE5HbC15cUpmMmtSYU1tamRDa185ZmdnOUlUMGItMzBQcGExSGZTVUNuNGQyVzJIcTczU1lseHU1ZkU3eXVVc3ltZTZmUjFoSDkydTFO?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46121.42167824074</v>
+        <v>46122.38089120371</v>
       </c>
     </row>
     <row r="3">
@@ -545,22 +545,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Amazon CEO says robotics is key for faster delivery, lower costs - The Robot Report</t>
+          <t>Amazon Pharmacy and Eli Lilly Launch Foundayo GLP-1 with Same-Day Delivery and Transparent Pricing - HLTH</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Amazon CEO says robotics is key for faster delivery, lower costs - The Robot Report</t>
+          <t>Amazon Pharmacy and Eli Lilly Launch Foundayo GLP-1 with Same-Day Delivery and Transparent Pricing - HLTH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 23:50:31 GMT</t>
+          <t>Fri, 10 Apr 2026 08:42:05 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOOWVLUnJwVXl2Wkp0RmhmUS1RNkJldVVHeENmTHpzdlhHaGFmcC1CdUNnc0NRb3I3cDFYNVRDVjBEMHVKOVVPNTBxMnBwbFcwREF2ME1uTVp3dXJ6R191R3hselpvWmpoSlYyVFEwUTN0Zi1EcWtrZEtOeTlMdkRncE1GcXc3MUJyWC1qVGRjVHFOUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxPemozZ2FMNlVMYVJHWEFKNlZHSDdkYkg5ZEJneWpQZUp1ODJKU25EZmMzbm8yRjdRTktmOXZtMGQxM3Nwa2pkSXJRMGp3X0Zyb1pkR1RyODllVTQycTd4NXM5N2J0RF9LZE12dXZSNXI3QVNFdE5VWEFIa2JxcnZZMlZ6OF9DTTdON01kSkxjdGxsX2U4aVY0OWRCLWdMNWhOdktUWC1wZ1NrVmNIUG92YnRCMHNlQnR2bEtSYlVQeXp5SHB2V0pQaGJ1M01lQjJncXB6c2RrSQ?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46121.99341435185</v>
+        <v>46122.36255787037</v>
       </c>
     </row>
     <row r="4">
@@ -600,22 +600,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Amazon Pharmacy to Offer Eli Lilly and Company’s New GLP-1 Pill Foundayo via Same-Day Delivery - Business Wire</t>
+          <t>Amazon CEO says robotics is key for faster delivery, lower costs - The Robot Report</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Amazon Pharmacy to Offer Eli Lilly and Company’s New GLP-1 Pill Foundayo via Same-Day Delivery - Business Wire</t>
+          <t>Amazon CEO says robotics is key for faster delivery, lower costs - The Robot Report</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 11:49:00 GMT</t>
+          <t>Thu, 09 Apr 2026 23:50:31 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxNcWhxU2h0ZEoxRFRwYVJPQm9zeUlIYTV5TmZFdEtBNHh6ZlB4SVBRUW5aRUwtVVNnZm15Wmg4QlFzYWFOQXFCWG5qSzRhMGVJT1A4YV9Wa3VBREVIYnQ0V3FXSFhsT2tnS3lNNmY0dm9jc0t1N2FYaVRSWjdhZVRZYk81OVNLMVVEVFlva3NYbk5MUy1RXzlUWEttUlZGZ0RDTVpHdEtZVy1QWkpWTkFLUnhBTTdnU1VMQkZUT2NQYkx4czRvU0w0TkJhRTgxTDF1VUdTSHJZZ2hhaHN3T2lRcGhId3c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOOWVLUnJwVXl2Wkp0RmhmUS1RNkJldVVHeENmTHpzdlhHaGFmcC1CdUNnc0NRb3I3cDFYNVRDVjBEMHVKOVVPNTBxMnBwbFcwREF2ME1uTVp3dXJ6R191R3hselpvWmpoSlYyVFEwUTN0Zi1EcWtrZEtOeTlMdkRncE1GcXc3MUJyWC1qVGRjVHFOUQ?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46121.49236111111</v>
+        <v>46121.99341435185</v>
       </c>
     </row>
     <row r="5">
@@ -655,22 +655,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Amazon and USPS agree to new terms for package delivery - Retail Brew</t>
+          <t>New Amazon center makes 1-hour delivery possible in Reno for first time - Reno Gazette Journal</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Amazon and USPS agree to new terms for package delivery - Retail Brew</t>
+          <t>New Amazon center makes 1-hour delivery possible in Reno for first time - Reno Gazette Journal</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 19:01:24 GMT</t>
+          <t>Thu, 09 Apr 2026 23:30:00 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOc2ZKRTNOd2JqeVZFczVPWVlsa0plWV9EUjVwbHppWmtlMDZtcVphak5fNW5PcHVQcTJrNG1aa3pGZG9VbEduVUgyU0hMYVR3WDhhUFAzdDQ3UElqbklOT2xLVXJ3VDhzUDh6VEhhWHB5UDNLNE0xdTRxWWUzZmt6V3dSaS0xZVVtOGpSY0JWTDdPTXB3SUpBQ1Y1NGk1SjRlOFZZ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPcWNkUFpNRTZ1dVI5ZFczOXN5NXVQdkRJRHJ3WXBNMkZLM2dVRmd6czQtMnJKSEJfcG9MWTlFZHYxdklTMHdYNmlOZGc2X2JkV29KNVpnREtvTzNVbnBETXcwczU5VHlaSGFiVHZlX08xMURBSW9XUFM5dXJ5UUtvYjF3dUd5ZWFJR2FGRFNEWnVsc0pWR1JJdlV5eU5SZDR4VDJxd25ZMU9ya00xZG5R?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46121.79263888889</v>
+        <v>46121.97916666666</v>
       </c>
     </row>
     <row r="6">
@@ -710,22 +710,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Amazon’s AI infrastructure is a limiting factor in supply — and that’s where the opportunity lies - Bitget</t>
+          <t>Amazon and USPS agree to new terms for package delivery - Retail Brew</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Amazon’s AI infrastructure is a limiting factor in supply — and that’s where the opportunity lies - Bitget</t>
+          <t>Amazon and USPS agree to new terms for package delivery - Retail Brew</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 15:52:24 GMT</t>
+          <t>Thu, 09 Apr 2026 19:01:24 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiY0FVX3lxTE1XUEU1aEFURnVLTm9qZVNoeVF1OVdPT1RJWl95Vnk0RmxPWEJINWx3VFdkSWlTREtua2M3WUJPSHVSRFVGZ2pFVGVuWEszOXdnNnBDMC1qVmFieHpCNjhIaTlNMNIBY0FVX3lxTE1XUEU1aEFURnVLTm9qZVNoeVF1OVdPT1RJWl95Vnk0RmxPWEJINWx3VFdkSWlTREtua2M3WUJPSHVSRFVGZ2pFVGVuWEszOXdnNnBDMC1qVmFieHpCNjhIaTlNMA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOc2ZKRTNOd2JqeVZFczVPWVlsa0plWV9EUjVwbHppWmtlMDZtcVphak5fNW5PcHVQcTJrNG1aa3pGZG9VbEduVUgyU0hMYVR3WDhhUFAzdDQ3UElqbklOT2xLVXJ3VDhzUDh6VEhhWHB5UDNLNE0xdTRxWWUzZmt6V3dSaS0xZVVtOGpSY0JWTDdPTXB3SUpBQ1Y1NGk1SjRlOFZZ?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46121.66138888889</v>
+        <v>46121.79263888889</v>
       </c>
     </row>
     <row r="7">
@@ -765,22 +765,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>New Amazon center makes 1-hour delivery possible in Reno for first time - Reno Gazette Journal</t>
+          <t>Amazon’s AI infrastructure is a limiting factor in supply — and that’s where the opportunity lies - Bitget</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>New Amazon center makes 1-hour delivery possible in Reno for first time - Reno Gazette Journal</t>
+          <t>Amazon’s AI infrastructure is a limiting factor in supply — and that’s where the opportunity lies - Bitget</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 23:30:00 GMT</t>
+          <t>Thu, 09 Apr 2026 15:52:24 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPcWNkUFpNRTZ1dVI5ZFczOXN5NXVQdkRJRHJ3WXBNMkZLM2dVRmd6czQtMnJKSEJfcG9MWTlFZHYxdklTMHdYNmlOZGc2X2JkV29KNVpnREtvTzNVbnBETXcwczU5VHlaSGFiVHZlX08xMURBSW9XUFM5dXJ5UUtvYjF3dUd5ZWFJR2FGRFNEWnVsc0pWR1JJdlV5eU5SZDR4VDJxd25ZMU9ya00xZG5R?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiY0FVX3lxTE1XUEU1aEFURnVLTm9qZVNoeVF1OVdPT1RJWl95Vnk0RmxPWEJINWx3VFdkSWlTREtua2M3WUJPSHVSRFVGZ2pFVGVuWEszOXdnNnBDMC1qVmFieHpCNjhIaTlNMNIBY0FVX3lxTE1XUEU1aEFURnVLTm9qZVNoeVF1OVdPT1RJWl95Vnk0RmxPWEJINWx3VFdkSWlTREtua2M3WUJPSHVSRFVGZ2pFVGVuWEszOXdnNnBDMC1qVmFieHpCNjhIaTlNMA?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46121.97916666666</v>
+        <v>46121.66138888889</v>
       </c>
     </row>
     <row r="8">
@@ -820,22 +820,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Amazon Teamsters Urge Passage of Delivery Protection Act in NYC Council Hearing - International Brotherhood of Teamsters</t>
+          <t>Amazon to expand quick commerce service Amazon Now in US, Europe - ET Retail</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Amazon Teamsters Urge Passage of Delivery Protection Act in NYC Council Hearing - International Brotherhood of Teamsters</t>
+          <t>Amazon to expand quick commerce service Amazon Now in US, Europe - ET Retail</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 15:00:00 GMT</t>
+          <t>Fri, 10 Apr 2026 07:14:35 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxPbjhxSEdpbWZPTlJwNW5zUmJpcVN2WHJfYVY2TF9EVEpDVzV0YnJlM2NuSmIzcjdMSzhSemY3ejV3dVplcGpITFBkTk45d0QyeElucmdoTWZ3NDF1UlVPUGZ0RENQbE13YnVnSlNKNjlUVDBTYjFQQnZpWHZ3c1lyWHBscGhzN3FCZ0RvQ285ME04d1Z3SW93YnJXd1NPbUVOdnh6eTBaeEQwb1BsVmc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxNM0VxZEhxSWJ0YWxLb3VHZEdWUTNNSVF5dHctdlk4LVFrS3NuY2NUSTFDajZXRXFHdk5FZHdzNzMtS1dfaDBieXdPRkVjMWZRN2hfMnBlNnpBSnBRZEplSzNVcEVzV2FLaDhLNmozS3p5TlJPVy1jSUtNWFBGdkpZWGhwNWJSZFRrVWlnbzNDZE1mVnl3ZHlKaFc2aWpWclM0WTFXWW9YMERPQl9panN0WVhHbEhBZ0hFS0liN3FlR3pPNWx4ZUtoOGZfM1RVXzduT0dVRXJHNkhwTUk?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46121.625</v>
+        <v>46122.30179398148</v>
       </c>
     </row>
     <row r="9">
@@ -875,22 +875,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Amazon Now: Revolutionizing Quick Commerce with Ultra-Fast Delivery - Devdiscourse</t>
+          <t>Amazon (AMZN) Stock Surges on Eli Lilly Weight-Loss Drug Partnership - MEXC</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Amazon Now: Revolutionizing Quick Commerce with Ultra-Fast Delivery - Devdiscourse</t>
+          <t>Amazon (AMZN) Stock Surges on Eli Lilly Weight-Loss Drug Partnership - MEXC</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 12:43:10 GMT</t>
+          <t>Thu, 09 Apr 2026 15:04:43 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxQSWdRUUNvY2pfaVRXaEJMUjVEYWFRZTBrU2E0dk1KZERDVllyLU05eGh5SFBkUFFuQ1hqWUpZQWtCWW1sQ0poREhNYk5GRVpvSzVqM1hCVzNUdnplOXhSeWxlb3JrTW5jeHBfR0tMVXpvUFR0OGd3NTl1aGVMWXBZQk8xSlhqaHRDUmxyUmZoYU43WDZxdGZZQjRkbndwalNLWTZqdWdsMGxCUDdXdWk4M3RnVWluZWNhOFRCcE1oTTRMUdIBwgFBVV95cUxQSWdRUUNvY2pfaVRXaEJMUjVEYWFRZTBrU2E0dk1KZERDVllyLU05eGh5SFBkUFFuQ1hqWUpZQWtCWW1sQ0poREhNYk5GRVpvSzVqM1hCVzNUdnplOXhSeWxlb3JrTW5jeHBfR0tMVXpvUFR0OGd3NTl1aGVMWXBZQk8xSlhqaHRDUmxyUmZoYU43WDZxdGZZQjRkbndwalNLWTZqdWdsMGxCUDdXdWk4M3RnVWluZWNhOFRCcE1oTTRMUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiSEFVX3lxTFBKYzlsZF9MZ1BSVFBPcGp2NFA0RUhjXzl4ZGpDNFpGQWRGRDhfOURTNTF2aW82dTVMMUw2VGZnUGZ4aDNhWTF3eg?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46121.52997685185</v>
+        <v>46121.62827546296</v>
       </c>
     </row>
     <row r="10">
@@ -930,22 +930,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Amazon Highlights Robotics, Rural Delivery and LEO Expansion - TipRanks</t>
+          <t>Amazon contractors clash with Teamsters at raucous NYC Council hearing on controversial delivery legislation - New York Post</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Amazon Highlights Robotics, Rural Delivery and LEO Expansion - TipRanks</t>
+          <t>Amazon contractors clash with Teamsters at raucous NYC Council hearing on controversial delivery legislation - New York Post</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 10:48:18 GMT</t>
+          <t>Thu, 09 Apr 2026 21:18:00 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPdEJWdFBlVE4wY3hhVzZ1Xzh6Y2JXRUdjSFNLVVRxc19zRldaYkE5WjN3Y1NQVmxwRUJLRkswSjVWLXJ1eFQ2ZTBKUndGQTVGQlEtNEswYWY1cUVvNDQ0Uy1EYVhJYm45dHJzcG5waWd0N2huUVB3dmVtZF9obVhWQkY1YlRZR3JMeUdjZnJhNkNEbnFHbEloQkszV2lISy15VHliYm05ZnVMWEtsdnNDUA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxPbzVUc2RmMjlrWEt6d0VwemJrX1lmNmI5Z2ZMQjRycWdFZ3k1RmxzbjVTZjdrRGlVYkhYUmgtMnNlb256RDNOTnUyS2tmTVdZOFJwREJHMG1aeml1b29FZFBCT0FTUWdUTFpEbGFuN1VvMWJWd1BuWU95ZEZHOUNwb2RBXzRMVWtpczRzekVvY091Nm1HZzRfTkk5QWJLNENicHVHenJhZk5qd0pHNEU2d1dtVllGbFlDV1JLeFJKX2puRkdtSFY0QVZEdi0yZktSM1g0d2RVQnpsOWN2bmZydzJn?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46121.45020833334</v>
+        <v>46121.8875</v>
       </c>
     </row>
     <row r="11">
@@ -985,22 +985,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Harris Farm Markets groceries now available for same-day delivery with Amazon Australia - Retail World Magazine</t>
+          <t>Amazon Now: Revolutionizing Quick Commerce with Ultra-Fast Delivery - Devdiscourse</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Harris Farm Markets groceries now available for same-day delivery with Amazon Australia - Retail World Magazine</t>
+          <t>Amazon Now: Revolutionizing Quick Commerce with Ultra-Fast Delivery - Devdiscourse</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 22:00:00 GMT</t>
+          <t>Thu, 09 Apr 2026 12:43:10 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQTVRjYWJaNGJEVE1Xbjk3YV9DVENoRUdWUjRJMGMwbldmUkNDMUVrdC1qWlJpTExLRkF5VVd5M0pGa1ZUVnc3bzA5RThETG5iZGNkYmoyLThNTjN4SkxZdzk0SnRCc2MxV3ppRmVkdTgzc0VKU1dhQlRGcWhXYURhS3lNWXdkdlpTaVlxOWsxeHNUdUtpWGhMdmhyQm41X01Dck5Vam5YU0FWQTFnSkx1TmJKWE9lNWpYcDZrWlVSczA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxQSWdRUUNvY2pfaVRXaEJMUjVEYWFRZTBrU2E0dk1KZERDVllyLU05eGh5SFBkUFFuQ1hqWUpZQWtCWW1sQ0poREhNYk5GRVpvSzVqM1hCVzNUdnplOXhSeWxlb3JrTW5jeHBfR0tMVXpvUFR0OGd3NTl1aGVMWXBZQk8xSlhqaHRDUmxyUmZoYU43WDZxdGZZQjRkbndwalNLWTZqdWdsMGxCUDdXdWk4M3RnVWluZWNhOFRCcE1oTTRMUdIBwgFBVV95cUxQSWdRUUNvY2pfaVRXaEJMUjVEYWFRZTBrU2E0dk1KZERDVllyLU05eGh5SFBkUFFuQ1hqWUpZQWtCWW1sQ0poREhNYk5GRVpvSzVqM1hCVzNUdnplOXhSeWxlb3JrTW5jeHBfR0tMVXpvUFR0OGd3NTl1aGVMWXBZQk8xSlhqaHRDUmxyUmZoYU43WDZxdGZZQjRkbndwalNLWTZqdWdsMGxCUDdXdWk4M3RnVWluZWNhOFRCcE1oTTRMUQ?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1024,7 +1024,7 @@
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46121.91666666666</v>
+        <v>46121.52997685185</v>
       </c>
     </row>
     <row r="12">
@@ -1040,22 +1040,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>The Ministry of Defense installs a giant photovoltaic plant and ensures a stable supply of clean energy in Maturacá, in the Amazon. - CPG Click Petróleo e Gás</t>
+          <t>Harris Farm Markets groceries now available for same-day delivery with Amazon Australia - Retail World Magazine</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>The Ministry of Defense installs a giant photovoltaic plant and ensures a stable supply of clean energy in Maturacá, in the Amazon. - CPG Click Petróleo e Gás</t>
+          <t>Harris Farm Markets groceries now available for same-day delivery with Amazon Australia - Retail World Magazine</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 11:35:00 GMT</t>
+          <t>Thu, 09 Apr 2026 22:00:00 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigJBVV95cUxQR0FZNHk0ZjQwdV8ycS04cFZUOF9XWXdyNi1rbG1vMVBqOTNqZnBpZGkxVGVWeVdNeWNkU2dyaTdzSDd4VERqaEVwLUhGeWZaS0k3QXNyN1Z1RW5QdWs5RGh3TVBFQURZdGVkckxSc05QSFI2dU1nMlNJMDZscU5rT3BnNmtJNk4yTVFJc1A2V2t4b19xY2FZMUlraDJMME5FekFqT3F6Yko0dFNLLTlnZXhQZ2ZTYkhZQUh6ekJIdzBrZFJYdTMzdDhrTlloUHh3Z3JYNE1GZmFlUENRdVVLeU84TndMdFlia2ozVElSWTZ0Z3FQRm5qNnY4WmhkMU9LdDFlVW4zd2ROUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQTVRjYWJaNGJEVE1Xbjk3YV9DVENoRUdWUjRJMGMwbldmUkNDMUVrdC1qWlJpTExLRkF5VVd5M0pGa1ZUVnc3bzA5RThETG5iZGNkYmoyLThNTjN4SkxZdzk0SnRCc2MxV3ppRmVkdTgzc0VKU1dhQlRGcWhXYURhS3lNWXdkdlpTaVlxOWsxeHNUdUtpWGhMdmhyQm41X01Dck5Vam5YU0FWQTFnSkx1TmJKWE9lNWpYcDZrWlVSczA?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1079,7 +1079,7 @@
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46121.48263888889</v>
+        <v>46121.91666666666</v>
       </c>
     </row>
     <row r="13">
@@ -1095,22 +1095,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Twee neven geven zich aan na schietpartij in Mechelen: slachtoffer (34) werd in been geschoten - GVA</t>
+          <t>Man (49) die explosie veroorzaakte in badkamer in Zutendaal blijft in de cel voor poging moord op zijn vrouw - Nieuwsblad</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Two cousins ​​turn themselves in after shooting in Mechelen: victim (34) was shot in the leg - GVA</t>
+          <t>Man (49) who caused explosion in bathroom in Zutendaal remains in jail for attempted murder of his wife - Nieuwsblad</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 15:55:00 GMT</t>
+          <t>Fri, 10 Apr 2026 11:28:49 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9gFBVV95cUxQRXdPZFYyNWJHbG9iajlLZFlocEpDSmRLT0xUMGFENnVYVWp2ci05RzFybThkQjV5S2huVzRPNGZlZGxNRl9IRldOR1p3UVpFMXlwbVh5NVJGMDRBUUR0MmY4QXM4MDVETXRXdzhLX0t6eHdqNzNaY0NvTFlHTi01bVBQczYxSDVhQ1Z0d0xMaTNXMmYtckFPVkxJWTdFSTd6ckhqZXRnZ1k4SnBScnhHVlBTOTRSSUpQRjhua2hSU2pSTzN6TmhHa2FjYUpuX2pEdXdzYnJfcGF5d19SUU1vcXNiSkw4OFpCb0Y0S0FjcWtIdWE1TkE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxObERYakQ2Vkh4UmRpVTM1QXl1NjFtcV9LTDN2VFhoSkVIclY4Z1ItLUxKUG9sWjExWFBxVWFVc1pPZkF2SzNUbEhtUlo1ZEJfdnhMa1ZjV25WR2Z3bW1lNjdlY092aXZuaXFNNHZWUkFjU1I1SmVVS3hSNC1UY2lxLUVtaFBXX1pnV2FjZXp4UlBlVnNQa1c1SVdtajNUajZPODRQUFpPbG1JbUNzVTE5WjM2Z0d6UlMwZ2ZYbzdaanh2MGNNRkdhZV9od0tuYWFaU3VwdllYaXVJeW1GMEFQcVpacGhja0JCR3JDbFBRVQ?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1134,7 +1134,7 @@
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46121.66319444445</v>
+        <v>46122.47834490741</v>
       </c>
     </row>
     <row r="14">
@@ -1150,22 +1150,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Aan cafés gelinkte bendes zorgen al jaar voor overlast in Van Kerckhovenstraat: gemiddeld vijf politie-interventies per week - Nieuwsblad</t>
+          <t>Dubbele liquidatie in Frankrijk: Nederlander (50) op straat doodgeschoten in rustig dorpje - HLN</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Gangs linked to cafés have been causing nuisance in Van Kerckhovenstraat for years: an average of five police interventions per week - Nieuwsblad</t>
+          <t>Double liquidation in France: Dutchman (50) shot dead on the street in a quiet village - HLN</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Fri, 10 Apr 2026 02:35:55 GMT</t>
+          <t>Fri, 10 Apr 2026 09:06:09 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiyAJBVV95cUxPTnRBNEhDS0h4Vk5jd25HUVdaZEFSd1JJdDlHamd3dzhnRXNSRFplZnBKeVJmal9kVVBqdmFsUXk2V3E3S3kzZlhsYTRkTUZVejRWTHVOTFFaa2RIWFFpV3VWb2lDdkdHY09Ycnhobm9rWm9NNEtWOUdBT2lBMjlOUXdKcWl2bzdoQ0JMTllQNXB3bGZRQnRZS3BoZGVpOEJxNGFObTRHdUx1TE5sSmMwZ3ZTa1hWaXpva29uenBaUVIzYml4WTZZX1NIWldtUHhYTzRwMDJBMDNuWEF6YUhINkF0Y2tJdUo4OUVSVXdsUnhMSzN0aE9tMDA0b2x0X1oyVEZidm9uWmJjMFl0cnlpNTVVWDBVcHdiWS1YOEYzOUZOS19mY0xGMFlpOWJtcFI3Mzk0dGtLT2xvc0c1V2hNWU0wcDNXVGNn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxNdzdudjZiU1VCd05pWF8yVDl5N1dPSW5ya1hwc29uQlRaNWhnaHJlODZQNzkwNkdJak02eVZ5OVpTS0hBWEFnWHE0STJEcEhFV3NuaEs1YWIwejVtV1Y5N25NRGZrMnlVQkhDS3M4VktDZ2pRZEs4NFJmWmNTM2tHU0VweGUycWpwMUpNV19EWjdBalZfWTI1Y3Q4RzRCaUh0c1A5YzNXZUpqdERRaGNhU2gzVWJWZ0RsdXhqVy1yVTQ5N1l5Mmc?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46122.10827546296</v>
+        <v>46122.37927083333</v>
       </c>
     </row>
     <row r="15">
@@ -1205,22 +1205,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Link met Oostende in Nederlands drugsonderzoek: negen verdachten opgepakt - HLN</t>
+          <t>Twee neven geven zich aan na schietpartij in Mechelen: slachtoffer (34) werd in been geschoten - GVA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Link with Ostend in Dutch drug investigation: nine suspects arrested - HLN</t>
+          <t>Two cousins ​​turn themselves in after shooting in Mechelen: victim (34) was shot in the leg - GVA</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 10:42:05 GMT</t>
+          <t>Thu, 09 Apr 2026 15:55:00 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOejFOVjJFdjlQUFpuQXlxMFF3UjhKTUFHUFBBUTZtTTRvc1hlR1dBRGNUSnhqdFc0NzdvRTN6ZGF6OGxqRHVsbzJsUFBpSHoyUXVlSkpoY1R6RmhUUFg5Sm9haEcxTklCNmNSa1p3WDhWQUNhMDJhMDZYcElCaWFSZnA4ejRrYldCRjZNUjVnZXg5X0d5RnoxQ3lGMzRyODVRMUlfV0JjZGJ1S1lwU0Nz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi9gFBVV95cUxQRXdPZFYyNWJHbG9iajlLZFlocEpDSmRLT0xUMGFENnVYVWp2ci05RzFybThkQjV5S2huVzRPNGZlZGxNRl9IRldOR1p3UVpFMXlwbVh5NVJGMDRBUUR0MmY4QXM4MDVETXRXdzhLX0t6eHdqNzNaY0NvTFlHTi01bVBQczYxSDVhQ1Z0d0xMaTNXMmYtckFPVkxJWTdFSTd6ckhqZXRnZ1k4SnBScnhHVlBTOTRSSUpQRjhua2hSU2pSTzN6TmhHa2FjYUpuX2pEdXdzYnJfcGF5d19SUU1vcXNiSkw4OFpCb0Y0S0FjcWtIdWE1TkE?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46121.4458912037</v>
+        <v>46121.66319444445</v>
       </c>
     </row>
     <row r="16">
@@ -1260,22 +1260,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Schietincident op Malpertuisplein Maastricht waarschijnlijk onderdeel van ripdeal. Maar wie wilde wie beroven? En wie was de schutter? - De Limburger</t>
+          <t>OM eist 28 jaar celstraf voor 11 jaar oude liquidatie: ’Legt pijnlijk bloot hoe over mensenlevens wordt gedacht binnen de Mocromaffia’ - Noordhollands Dagblad</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Shooting incident on Malpertuisplein Maastricht probably part of rip deal. But who wanted to rob whom? And who was the shooter? - The Limburger</t>
+          <t>Public Prosecution Service demands 28 years in prison for 11-year-old liquidation: 'Painfully exposes how people think about human lives within the Mocromafia' - Noordhollands Dagblad</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 10:49:03 GMT</t>
+          <t>Fri, 10 Apr 2026 10:52:08 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAJBVV95cUxPV0RSWDV4NVRrNXZBVFJ1YlFzUUpmX1ZfQVVkc0w2dXVBRXdHZ0lWQWRLRHZIS3VrOWQ2TVgwTW8xOHc3dW1qOUtLak9xeWlmcVV3LWVSUnFodm9fQjEwX29IclpnTlBIUXBJNmhpRWI1Q2pIOGZGMTNmbkZXX3BqeEcyUmlMMk5LUnNlMTZEZDRnYjhPVXcxQUZEU0syMnkydGRjNGlwVUdsX3FrMDBLOEpsWWhqMU8xV192eGpQYjNTdG9TcW1yWXFpQ2tUcFBxMVN6RmM4Ykh5WndmdGgxVW5Qb2F5UEM1eHVVbVNXMUZNY2s5dmpxZE0wTnAwSUhxelpBVW5FZkczUjdoUlA2RGR1TFVRM1ho?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgJBVV95cUxQbTlJTWIyVkd0UGZMOEg5SGNIRjVleTFDZW9LR2poTzZ1WXVrNHpGczZ5eDk5ZEUzclI2TTEyQnQteW9rS1VHdGxoWGpnRG8wRVJnWTZUdlFYNWtRSGw1WXp5YkZ6QWp4YVFfYk54S080SHNxaUdFWTkzY3RaM29HMF96TlM2RzNYd0tGMGV6SHdEWEJJUlpnQWRzcG5MNlhtRGQ4Y053TUNvY2RVUG1EcHlyUk9yVWRTN0VYTHVqeHFFS0MzV3BOMUhvUmlDNVZWbHZyNDFvNUxMR1MySHB6b1R6bW9oMEw4UnE2VE9FYUU3NHh6eHlLS3hUX21sanJYRk5OYnljQkVXVEJSZTZmS1h2MG5RN1dnT1c3YXA4VmROVGFPMGd0ekROMllNekkzSWtybnpYSlphdHRLcklJem9B?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46121.45072916667</v>
+        <v>46122.45287037037</v>
       </c>
     </row>
     <row r="17">
@@ -1315,22 +1315,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Twee verdachten voor schietpartij in Battel aangehouden: “Ze kwamen zichzelf aangeven” - Nieuwsblad</t>
+          <t>Aan cafés gelinkte bendes zorgen al jaar voor overlast in Van Kerckhovenstraat: gemiddeld vijf politie-interventies per week - Nieuwsblad</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Two suspects arrested for shooting in Battel: “They came to turn themselves in” - Nieuwsblad</t>
+          <t>Gangs linked to cafés have been causing nuisance in Van Kerckhovenstraat for years: an average of five police interventions per week - Nieuwsblad</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 14:17:29 GMT</t>
+          <t>Fri, 10 Apr 2026 02:35:55 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxPSVNGcC10bjV4eGN6a3YwRUhRZlEyWWx1REFpQVBiU0RjR0lYZmhaVm12elJqZzBHWm1vdTlKbVVXMWZPS2h1SEZTNnd0U21LQXc4a29mM2phWG5PX1BqUFJNUEZMWVo0VlB4UGhKM245bS1iRHA0Rl9Mcm1oekZleEVhTU01ZUdnNG5qSG5xZXdNT0ZwS3FtQkRJTm10Z2hLWlNnNGxrZ0FEZXpEXzhodFZsdktZd2swcFNnTjVyNnB5c3lvRmtJamF2b2ZMYlFLNnJUTFFwVzQyNjVxQVpVUmVOZGtKRTNiV3RWMWVVVVFPakhL?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiyAJBVV95cUxPTnRBNEhDS0h4Vk5jd25HUVdaZEFSd1JJdDlHamd3dzhnRXNSRFplZnBKeVJmal9kVVBqdmFsUXk2V3E3S3kzZlhsYTRkTUZVejRWTHVOTFFaa2RIWFFpV3VWb2lDdkdHY09Ycnhobm9rWm9NNEtWOUdBT2lBMjlOUXdKcWl2bzdoQ0JMTllQNXB3bGZRQnRZS3BoZGVpOEJxNGFObTRHdUx1TE5sSmMwZ3ZTa1hWaXpva29uenBaUVIzYml4WTZZX1NIWldtUHhYTzRwMDJBMDNuWEF6YUhINkF0Y2tJdUo4OUVSVXdsUnhMSzN0aE9tMDA0b2x0X1oyVEZidm9uWmJjMFl0cnlpNTVVWDBVcHdiWS1YOEYzOUZOS19mY0xGMFlpOWJtcFI3Mzk0dGtLT2xvc0c1V2hNWU0wcDNXVGNn?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1354,7 +1354,7 @@
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46121.59547453704</v>
+        <v>46122.10827546296</v>
       </c>
     </row>
     <row r="18">
@@ -1370,22 +1370,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Met duizend blinkende oldtimers: Antwerp Classic Car Event keert terug naar de kaaien - Nieuwsblad</t>
+          <t>Man zwaargewond bij steekpartij in winkelstraat Best, dader vlucht op e-bike - Studio 040</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>With a thousand shiny vintage cars: Antwerp Classic Car Event returns to the quays - Nieuwsblad</t>
+          <t>Man seriously injured in stabbing in Best shopping street, perpetrator flees on e-bike - Studio 040</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 14:44:19 GMT</t>
+          <t>Fri, 10 Apr 2026 08:01:47 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxQeDdyY0ZteGFvNzV0MmV6d3dleUp2dUhRNm1KakFCUmN4Yjg4anBwbE00ZDRUdmtvdUhGaU4tSkhKMkVqMzFQTlRzZzBZLVdlaHF5dk1Pd0FfSHF5NTNQQ0Q2T3p6cFFmT1prUHhMR3UzRmVMRFRuc0hzYzMxZXJLbTNjWWt4czBDaDh4b0diSjVXQl9aTEtzN0hxaEFYYnBpWVpUdXRmRGJoaW1HdU14UEIwU1VHb0RCRWpHb0JJcXBjX1ZGb3YwY0hxSXdoMkpZVFFVdXNRVmpYMi13SkdMMG5Fb3lzS3NqTzl1a1pCakMzaktmdVBTbFlJYw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxQR0xkVjd4ZnNuUG5MYzVLRDVLT0tLdUF0Mk5CLW1pZ2lpOHctWVdHSDB5TGZVNVdsWXA0bm5ZWTBhU2NWVGpVYlNkeVBaLXBxV0FBbUI5ZnJuRVlpMGJmMlNGRVFaMTJZQkloQUd6cmdfZ0hEZ3Zrd3RpaFBUQnNQaktDUjF2QmFNQ1pGdw?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1409,7 +1409,7 @@
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46121.6141087963</v>
+        <v>46122.33457175926</v>
       </c>
     </row>
     <row r="19">
@@ -1425,22 +1425,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Fietsers botsen langs kanaal in Olmen: 55-jarige vrouw zwaargewond - Nieuwsblad</t>
+          <t>Twee verdachten voor schietpartij in Battel aangehouden: “Ze kwamen zichzelf aangeven” - Nieuwsblad</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Cyclists collide along a canal in Olmen: 55-year-old woman seriously injured - Nieuwsblad</t>
+          <t>Two suspects arrested for shooting in Battel: “They came to turn themselves in” - Nieuwsblad</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 14:44:42 GMT</t>
+          <t>Thu, 09 Apr 2026 14:17:29 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxNMjlLYXlnSzlFM1l1ZmZYVHVoTzNPZm1kUng5VUEwSkFzY0R6bHVaa2wya1Q3dmc0bTJrb3BxTXg4NkRIRGlIYmRuTEdiSVgxYXZoUjBGb0hfSDJ6RFUtYXZwdkpLVFdSUDdJUi1UU0dTc3QxSG5VRzFadVpvTzNwbnVac1N0OFRadUIzeXdRaEozNlUwNzg4MUM1bWVrWGRLaXQ2M0RQTW8zOEhsSGYwMEozdkFOYklUTGJoV2VKcHlyYzhaeHI1WEZtMWc4LVA3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxPSVNGcC10bjV4eGN6a3YwRUhRZlEyWWx1REFpQVBiU0RjR0lYZmhaVm12elJqZzBHWm1vdTlKbVVXMWZPS2h1SEZTNnd0U21LQXc4a29mM2phWG5PX1BqUFJNUEZMWVo0VlB4UGhKM245bS1iRHA0Rl9Mcm1oekZleEVhTU01ZUdnNG5qSG5xZXdNT0ZwS3FtQkRJTm10Z2hLWlNnNGxrZ0FEZXpEXzhodFZsdktZd2swcFNnTjVyNnB5c3lvRmtJamF2b2ZMYlFLNnJUTFFwVzQyNjVxQVpVUmVOZGtKRTNiV3RWMWVVVVFPakhL?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1464,38 +1464,38 @@
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46121.614375</v>
+        <v>46121.59547453704</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>High Level City Belgium English (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>A view from Brussels: A European view from IAPP Global Summit 2026 - IAPP</t>
+          <t>Met duizend blinkende oldtimers: Antwerp Classic Car Event keert terug naar de kaaien - Nieuwsblad</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>A view from Brussels: A European view from IAPP Global Summit 2026 - IAPP</t>
+          <t>With a thousand shiny vintage cars: Antwerp Classic Car Event returns to the quays - Nieuwsblad</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 16:33:06 GMT</t>
+          <t>Thu, 09 Apr 2026 14:44:19 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxNQk9SYjk4ZVA5NnllUS1paUdKY2hORTdrdzJGbllNZUFtLURZUi10WHBKODRNc016WXd3a0xpVUFrSFFJai05em4yNGhabHV5bENERUttUm1uemUxSzI0T3VneWNELWRiZlRCNXJ4RWV4MFphd1V5YXl0b0dHVWlhMVVwcG1JN2s0bjU0bXRNZ2lFMTA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxQeDdyY0ZteGFvNzV0MmV6d3dleUp2dUhRNm1KakFCUmN4Yjg4anBwbE00ZDRUdmtvdUhGaU4tSkhKMkVqMzFQTlRzZzBZLVdlaHF5dk1Pd0FfSHF5NTNQQ0Q2T3p6cFFmT1prUHhMR3UzRmVMRFRuc0hzYzMxZXJLbTNjWWt4czBDaDh4b0diSjVXQl9aTEtzN0hxaEFYYnBpWVpUdXRmRGJoaW1HdU14UEIwU1VHb0RCRWpHb0JJcXBjX1ZGb3YwY0hxSXdoMkpZVFFVdXNRVmpYMi13SkdMMG5Fb3lzS3NqTzl1a1pCakMzaktmdVBTbFlJYw?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1515,42 +1515,42 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46121.68965277778</v>
+        <v>46121.6141087963</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>High Level City Belgium English (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>This Sunday, Hungary defines: Trump or Brussels - MVNU</t>
+          <t>Fietsers botsen langs kanaal in Olmen: 55-jarige vrouw zwaargewond - Nieuwsblad</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>This Sunday, Hungary defines: Trump or Brussels - MVNU</t>
+          <t>Cyclists collide along a canal in Olmen: 55-year-old woman seriously injured - Nieuwsblad</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Fri, 10 Apr 2026 04:39:59 GMT</t>
+          <t>Thu, 09 Apr 2026 14:44:42 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQVWxmd2k3bW5qbnJMRko5VVpvdThjQmk0Vy1UOWo2Tk44S0pMMkRnejJDazBrTXZmbHNxbDlXXzJGYzAtalFxTEdrdVZUYTFraHlOVlRJeVUzN3EwOGNoQzhkVHpkQ0M0Uk9NOGd1UWxYRUhTSlQxZ3FQWkZRS29JLQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxNMjlLYXlnSzlFM1l1ZmZYVHVoTzNPZm1kUng5VUEwSkFzY0R6bHVaa2wya1Q3dmc0bTJrb3BxTXg4NkRIRGlIYmRuTEdiSVgxYXZoUjBGb0hfSDJ6RFUtYXZwdkpLVFdSUDdJUi1UU0dTc3QxSG5VRzFadVpvTzNwbnVac1N0OFRadUIzeXdRaEozNlUwNzg4MUM1bWVrWGRLaXQ2M0RQTW8zOEhsSGYwMEozdkFOYklUTGJoV2VKcHlyYzhaeHI1WEZtMWc4LVA3?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1570,42 +1570,42 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46122.19443287037</v>
+        <v>46121.614375</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>High Level City Belgium English (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Wild animals and wilder friends: Viktor Orbán’s Brussels legacy - politico.eu</t>
+          <t>Motorrijder (42) uit Brunssum overleden bij ongeval in Maastricht - StadIndex</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Wild animals and wilder friends: Viktor Orbán’s Brussels legacy - politico.eu</t>
+          <t>Motorcyclist (42) from Brunssum died in accident in Maastricht - StadIndex</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Fri, 10 Apr 2026 02:01:37 GMT</t>
+          <t>Thu, 09 Apr 2026 14:45:12 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNaEZEeHRQSHo0TDNFM3laY0h6dDNjRHEyd1A5VlpYLVJweEYyazBQMEw5amoxOXc0WUE4dGJyQWk5eDdhbkl3d0g4NTV0N3MyeUlEakd6NU5fc3U4SDZ0UkVFZkhQaUlpNklZNTFtckRlMFdYbTUtVV92c0hzRnJkZnJYbXdseWlSY2NlUGhMVElpRTJwb3ltTW84VkttWjNlbkE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPeU51LUhVbHYwRjl5QzB5YWdMbnJuZE0ycFkta2Fxa3BmY0Y1MUFDSGRFcDlUWFByRUk3T1FGUmozWlpjWXd6N0VhQzhHZEg2UWVXRDJTd0R0bkJ2VHIwYzZTQXRJLUc1QjF5RFZHRGVXdVY5VTlQVGhyNlpMckR1LW1hNmtoMXJpVEdrMWpBWE9BT0FURDhHeW9uOTh6cUJtemExbnFCTmdLUVU?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,7 +1615,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1625,11 +1625,11 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46122.08445601852</v>
+        <v>46121.61472222222</v>
       </c>
     </row>
     <row r="23">
@@ -1645,22 +1645,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Taylor Farms Launches Additional Veggie Kit Flavors, Expands Brussels Sprouts Offerings - AndNowUKnow</t>
+          <t>Shipping traffic around Antwerp port partially halted after oil spill - Reuters</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Taylor Farms Launches Additional Veggie Kit Flavors, Expands Brussels Sprouts Offerings - AndNowUKnow</t>
+          <t>Shipping traffic around Antwerp port partially halted after oil spill - Reuters</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Fri, 10 Apr 2026 04:10:56 GMT</t>
+          <t>Fri, 10 Apr 2026 07:15:24 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxOYTdnSGNhQ05KU1JkdFZxUkQ0WG9QX09DRjBBQ2pYaWxxUmhZdnk5djlpcVdMQXhoeU1ZZ19DTV9vbUNJSmhYR0NmUk84aU1VdjhScWVZMkNVNlF6a1c1NVlGaDFrUEtVbUFWSkVZbEFKazZBMGJQdmZPREM3NmRWbVpLckNxN1E4REhZa2FHeGhOenpUZHFmbXF0TDVPSWd2VlpvUUo4ZkV5U3hGaVZFb2Rnc1M4a3NPMVdsREJscHpFSEtBODVJ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxNdWN4VC1nd1ZrYmZIMVp1cGg0a2hmWkRYNUNqMFl6bV9yeEd5d2NkMlBPN1ZGLXNkekxDNnpuWnM4cVNqcXphM2VfOVh1eko4VW5ockZDd3FCQ1dST1lJbnNaeTFhOTJobE5tR0FOb2dDbU5SN3BidlZobnh2R1NKZUU4SlBkaGFnRUxDSTNJbjZSWVI3cXhRYXVIM2dCOEptSjFMRXJYV3dVQW5WT2Jtag?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1684,7 +1684,7 @@
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46122.17425925926</v>
+        <v>46122.30236111111</v>
       </c>
     </row>
     <row r="24">
@@ -1700,22 +1700,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Antwerp’s CARROSER turn classical training into posthardcore tension on new EP - IDIOTEQ.com</t>
+          <t>Brussels Calling: First Ukrainian-language vodcast by DW - DW</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Antwerp’s CARROSER turn classical training into posthardcore tension on new EP - IDIOTEQ.com</t>
+          <t>Brussels Calling: First Ukrainian-language vodcast by DW - DW</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Fri, 10 Apr 2026 06:00:15 GMT</t>
+          <t>Fri, 10 Apr 2026 08:27:25 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeFcwVWtSaXRESU1qY190NHA1ZnBmQ0JnQjZpNEc5ZjFYNFRtRmFzZm9jY2UwdU5NZ3lEXzZObWNDRjNqaDhFSHJJME81M3JXYmlqTnI4ZTllbXBlcVl2dVNaRllQU2VUN3BhejdmM3JXWUpXN0xKZG5xLXZWRlVUdjRydUtFdTRFcW51SUM1b2lIN2FUYXRCSWhWbmpSQ1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxOM0xoelFXYWpSbE5YallSZklvbzZZOHhpRG1MYmgzYXRqd0FiNnFDNWo0dlg1RUE0bnJoRnlfSEllancxek54dDg5ZkQ5QlpUWkR0dVlEOVVKZWk5VFFYVW9hSnZ2LTk1aklqZ2YtUEdDY3NQdDdKZHg4UkhWYUFXNTBGUF9SWGFMRlJwa1FDZnljZTRpV2hlS0dFX1lTUVU5Ynd5a3Eyaw?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1739,7 +1739,7 @@
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46122.25017361111</v>
+        <v>46122.35237268519</v>
       </c>
     </row>
     <row r="25">
@@ -1755,22 +1755,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Most Hungarians want better relations with EU after years of Orbán Brussels-bashing, poll finds - The Guardian</t>
+          <t>Royal Charleroi vs. Antwerp (10 Apr, 2026) Live Score - ESPN</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Most Hungarians want better relations with EU after years of Orbán Brussels-bashing, poll finds - The Guardian</t>
+          <t>Royal Charleroi vs. Antwerp (10 Apr, 2026) Live Score - ESPN</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Fri, 10 Apr 2026 01:31:00 GMT</t>
+          <t>Fri, 10 Apr 2026 08:09:37 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPRUtOa1hGa1ZkdTUxeUFQVFRKUGVPckRuNTZSVzRLUWdUSnZKS2lobVVNUXgzZEo2LUxFQ1B3X3FNa1dNcGdyRmNqX085N29XME1YTlpTR0ljakhOdm5janpYLVFaTkZKa2ZheE5qMWZyRnlhb1Y5VDQ0NUJUcGZOMXdBalZNbVBDMzBHNDJ0Ri1jVnAzZmtFMzl3dXNGQ3BSWFRua1p2eXhmbkVJNzJNWUdoSzhHTmNVRmgyQzhLUGpHdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxQM2oxaVg1WDRWTlpTUTVIaUh0M2R0OEJpQlNtTzNZM2hOYnl4Um5xVjBQNDd3OFBOcmoyUlNmRzJqbUVtTllfNUJLRGZDNXV1T3g4MTlGTEZSSFh0SU1JQldsdFhHRGFoS0lpOUtPU0w2RUdpdEI4QlBwc1JwV3o4WHJxUkFKRHQ2aTVVag?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1794,7 +1794,7 @@
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46122.06319444445</v>
+        <v>46122.34001157407</v>
       </c>
     </row>
     <row r="26">
@@ -1810,22 +1810,22 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>International beer culture meets in Brussels - Brauwelt</t>
+          <t>Taylor Farms Launches Additional Veggie Kit Flavors, Expands Brussels Sprouts Offerings - AndNowUKnow</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>International beer culture meets in Brussels - Brauwelt</t>
+          <t>Taylor Farms Launches Additional Veggie Kit Flavors, Expands Brussels Sprouts Offerings - AndNowUKnow</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Fri, 10 Apr 2026 01:19:14 GMT</t>
+          <t>Fri, 10 Apr 2026 05:01:26 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOR3psMGtaUWhVak1vaXF0ejZSSWdTMVFsZF9kWERwTjBLY2dMUk9QVVl2dWJQVENBVWZpeVJuWmEtRk5ockotV1AtR3Zua1RESUFmXzgtTzBWS3owSTVNSHBGMGV5TmFpaGxzb1VWWVJnMUlUc01HLVR4aWtNa3Bha21EYTcyaGc4a0FHeWdKS200Q3JXamc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxOYTdnSGNhQ05KU1JkdFZxUkQ0WG9QX09DRjBBQ2pYaWxxUmhZdnk5djlpcVdMQXhoeU1ZZ19DTV9vbUNJSmhYR0NmUk84aU1VdjhScWVZMkNVNlF6a1c1NVlGaDFrUEtVbUFWSkVZbEFKazZBMGJQdmZPREM3NmRWbVpLckNxN1E4REhZa2FHeGhOenpUZHFmbXF0TDVPSWd2VlpvUUo4ZkV5U3hGaVZFb2Rnc1M4a3NPMVdsREJscHpFSEtBODVJ?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1849,7 +1849,7 @@
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46122.05502314815</v>
+        <v>46122.20932870371</v>
       </c>
     </row>
     <row r="27">
@@ -1865,22 +1865,22 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Brussels finds humor amid online clamor - China Daily</t>
+          <t>Wild animals and wilder friends: Viktor Orbán’s Brussels legacy - politico.eu</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Brussels finds humor amid online clamor - China Daily</t>
+          <t>Wild animals and wilder friends: Viktor Orbán’s Brussels legacy - politico.eu</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Fri, 10 Apr 2026 01:15:00 GMT</t>
+          <t>Fri, 10 Apr 2026 03:00:00 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1wSW0yYlR2MTUyXzNya3hWMlhfMHlVQWZQQzE0TTVROTRoQXJHcDUwVlZyb2M1VnBJN0R6VHdzQi0tSW50VHRZaWwzVko3ZW1pSVpEeWJxaW5sVlhFeHBJY2FnRWxqTmxyUl9TWmJmZDhwVmtDUU9icHhkb3hYQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNaEZEeHRQSHo0TDNFM3laY0h6dDNjRHEyd1A5VlpYLVJweEYyazBQMEw5amoxOXc0WUE4dGJyQWk5eDdhbkl3d0g4NTV0N3MyeUlEakd6NU5fc3U4SDZ0UkVFZkhQaUlpNklZNTFtckRlMFdYbTUtVV92c0hzRnJkZnJYbXdseWlSY2NlUGhMVElpRTJwb3ltTW84VkttWjNlbkE?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1904,7 +1904,7 @@
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46122.05208333334</v>
+        <v>46122.125</v>
       </c>
     </row>
     <row r="28">
@@ -1920,22 +1920,22 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Shanyraq Fest Brussels showcases Kazakh heritage in Belgium - Qazinform</t>
+          <t>This Sunday, Hungary defines: Trump or Brussels - MVNU</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Shanyraq Fest Brussels showcases Kazakh heritage in Belgium - Qazinform</t>
+          <t>This Sunday, Hungary defines: Trump or Brussels - MVNU</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Fri, 10 Apr 2026 03:58:57 GMT</t>
+          <t>Fri, 10 Apr 2026 04:39:59 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQcUhzWjRISG1CYnV4ejc3elN6LUltZkUycUtBMTF1V0Z3SG9ibVo3Rm5STVRrZFBuZTdzRmtDbTBWV2ZMOUpsMGZnTGpSVDNsR2lrX0pjbUdlSlNyZW9oWFZJeVJvM0pPOVFBdHFaQUdFNDNTNHR0Z0VKdllrejdSc2FtT2tCQlZIcWNQZzE5SGNoVndfLU00YdIBmAFBVV95cUxQcUhzWjRISG1CYnV4ejc3elN6LUltZkUycUtBMTF1V0Z3SG9ibVo3Rm5STVRrZFBuZTdzRmtDbTBWV2ZMOUpsMGZnTGpSVDNsR2lrX0pjbUdlSlNyZW9oWFZJeVJvM0pPOVFBdHFaQUdFNDNTNHR0Z0VKdllrejdSc2FtT2tCQlZIcWNQZzE5SGNoVndfLU00YQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQVWxmd2k3bW5qbnJMRko5VVpvdThjQmk0Vy1UOWo2Tk44S0pMMkRnejJDazBrTXZmbHNxbDlXXzJGYzAtalFxTEdrdVZUYTFraHlOVlRJeVUzN3EwOGNoQzhkVHpkQ0M0Uk9NOGd1UWxYRUhTSlQxZ3FQWkZRS29JLQ?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1959,7 +1959,7 @@
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46122.1659375</v>
+        <v>46122.19443287037</v>
       </c>
     </row>
     <row r="29">
@@ -1975,22 +1975,22 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Ukrainians evicted from community centre as Brussels axes funding - Euractiv</t>
+          <t>Orbán Is Very Much on the Right Track in Standing up to Brussels — An Interview with Tony Abbott - Hungarian Conservative</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Ukrainians evicted from community centre as Brussels axes funding - Euractiv</t>
+          <t>Orbán Is Very Much on the Right Track in Standing up to Brussels — An Interview with Tony Abbott - Hungarian Conservative</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Fri, 10 Apr 2026 04:02:34 GMT</t>
+          <t>Fri, 10 Apr 2026 10:00:58 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNVW9oMGd3NFJHU3BFRGpQSC1LWWV6cC1ibVVJcExNWkprMTVGY3lGRzZoLXV2ZmUxbllsTjB1SGlWbGVvY1ZuNVM3WmYyd1NSdVVkZlZUekxLT0RQd1dKX0ZFQy1NVTVGU2lIR0dpaG5vQ1RNY1VTbmE3bmZ4SWo4QlJOVGtWaklsWk1PZ285YjM5UWNaWGFEUVNNUWw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOM0Y5T2F5N0twb1FiaVQ5bjNQRHlJQXhELThEbFZzS1V4eFZGNDJpT3hyM3hDcTNtWnNaSDFfZEtxOWxRMzRnaFRWbzBDRXpPd0RBN2pNempFdUw4YWM5cHVPVDJIQjhMNl9FRUdCS3N6NDFtU3NYTTFCRm96dXVlRnBsLXB5UHgxRDlhX3p2N0s2ZzFobzdqdC1wZ3F3bmF1S0JEUA?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2014,7 +2014,7 @@
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46122.16844907407</v>
+        <v>46122.41733796296</v>
       </c>
     </row>
     <row r="30">
@@ -2030,22 +2030,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>One Fine Show: “Bellezza e Bruttezza” at Bozar in Brussels - observer.com</t>
+          <t>A view from Brussels: A European view from IAPP Global Summit 2026 - IAPP</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>One Fine Show: “Beauty and Ugliness” at Bozar in Brussels - observer.com</t>
+          <t>A view from Brussels: A European view from IAPP Global Summit 2026 - IAPP</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 13:20:35 GMT</t>
+          <t>Thu, 09 Apr 2026 16:33:06 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPc3dYamNsZEM4U2YtRWtmNW9ia3VNNG1waUZhTkhRTzR1Q3ZhQTBXeVlrNzZKNVhkekYyWWFxTmxDU1hlbFFSN3pXZHhzSV9ZTE1ZenRKT0Q3ZTZZTnVub2FweS1VQlhXWF8tZzJLMnFKSmhSWnp5QmtaOG9mQk1aT3FTUGphOWVWWGFiMkV1UHVPcUJkUHdfN1FR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxNQk9SYjk4ZVA5NnllUS1paUdKY2hORTdrdzJGbllNZUFtLURZUi10WHBKODRNc016WXd3a0xpVUFrSFFJai05em4yNGhabHV5bENERUttUm1uemUxSzI0T3VneWNELWRiZlRCNXJ4RWV4MFphd1V5YXl0b0dHVWlhMVVwcG1JN2s0bjU0bXRNZ2lFMTA?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2069,7 +2069,7 @@
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46121.55596064815</v>
+        <v>46121.68965277778</v>
       </c>
     </row>
     <row r="31">
@@ -2085,22 +2085,22 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Fact-checking JD Vance's claims that Brussels is 'harming Hungary' - Euronews.com</t>
+          <t>Antwerp’s CARROSER turn classical training into posthardcore tension on new EP - IDIOTEQ.com</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Fact-checking JD Vance's claims that Brussels is 'harming Hungary' - Euronews.com</t>
+          <t>Antwerp’s CARROSER turn classical training into posthardcore tension on new EP - IDIOTEQ.com</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 15:00:07 GMT</t>
+          <t>Fri, 10 Apr 2026 06:00:15 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxOcmdaWEJvYTdUNmJzQXZMcnlSbjU5TndCaHFzMjkxSVRjd0dibnlXSW9vWnI5NUR2TnVzd3F6dUVfdW5PQ0N3NEZPSFh2QmFPWE1mMUlLWThJSFdCNXRQUkhoVTlzdU5zcFJnQ3ZNOGRXVmpqSDFmdVJwQTM0NUo4X2V4Nzk4TGFjNXN3ak1XZG1kdjgyNHZJMFc0Rks4TXA5ZEZNTzBHOEYycGdJVnc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeFcwVWtSaXRESU1qY190NHA1ZnBmQ0JnQjZpNEc5ZjFYNFRtRmFzZm9jY2UwdU5NZ3lEXzZObWNDRjNqaDhFSHJJME81M3JXYmlqTnI4ZTllbXBlcVl2dVNaRllQU2VUN3BhejdmM3JXWUpXN0xKZG5xLXZWRlVUdjRydUtFdTRFcW51SUM1b2lIN2FUYXRCSWhWbmpSQ1E?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2124,7 +2124,7 @@
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46121.62508101852</v>
+        <v>46122.25017361111</v>
       </c>
     </row>
     <row r="32">
@@ -2140,22 +2140,22 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>At Waterstones Brussels, Ipek Tekdemir makes the case for trust in an age of noise - EU Today</t>
+          <t>Ryanair flight FR4523 is declaring an emergency after go around at Brussels Charleroi Airport - airlive</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>At Waterstones Brussels, Ipek Tekdemir makes the case for trust in an age of noise - EU Today</t>
+          <t>Ryanair flight FR4523 is declaring an emergency after go around at Brussels Charleroi Airport - airlive</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Fri, 10 Apr 2026 06:30:17 GMT</t>
+          <t>Fri, 10 Apr 2026 08:05:11 GMT</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPaFFvcHlIVHQtY2ROMHp1QUs2RW4wUDBULThQdVZnWC1KWGQ0MmJ0Wk9IYlhzR1BpeGRjY0YwS1BQMlVMVU1jdWN0ZExGNG5KRXVJRTJNaGFzeERiOTdwX2dSV3BSbVRFRXVFX3dUWW1ZQTNZeFdSa1JPeDZtZ1dlT0FLcTZNTG1hZWw4N3NCMHFOV0tXd25ZLWhoMkdTbnVBUWpHUg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxPcHFKSFU2WWRCVGdVdnhvOHdqQlQ1al9ieFgzQUo2N2NqdzBibVNiUU50b0I5MEV5cGc5S09kdDVRa0pNQVBTUTZqMmR0dDEyYjcyTWVEa3Vrb1FmSURsaWZtY1dFX2xPYUZOY3JuVVRvVDlJbUI2OGh4YkE1RnV5YU5WbE02QWw2R1F3MkNPenFwTDBDU0RWcXpHdE5BZEs4UGJ6WC1lR0pnbUY5cDV0ZkRFYnZhTno4UWNjZHpFc1RPeHpOa0tXUnkxMG5jOTdU?oc=5</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2179,7 +2179,7 @@
         </is>
       </c>
       <c r="K32" s="1" t="n">
-        <v>46122.27103009259</v>
+        <v>46122.33693287037</v>
       </c>
     </row>
     <row r="33">
@@ -2195,22 +2195,22 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Trust in EU grows in Southeast Asia, but challenges remain - dw.com</t>
+          <t>Most Hungarians want better relations with EU after years of Orbán Brussels-bashing, poll finds - The Guardian</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Trust in EU grows in Southeast Asia, but challenges remain - dw.com</t>
+          <t>Most Hungarians want better relations with EU after years of Orbán Brussels-bashing, poll finds - The Guardian</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 20:53:03 GMT</t>
+          <t>Fri, 10 Apr 2026 01:31:00 GMT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxPcDc2MFFrOGV4SUw2VFlMbnFtVE5BSDR5QlJrUGlXVVNpZzJUQ2ltRnBtZ1A5WWtKaGRJVERrci1MWWVrb0NKRDNrYmprNFpiR0p2Z182WFExT19zcHJHdGVPcjFjSGtkbWZTLXpBVXlINS1wOG05OGtnQ05lSGZneEtEOURYV3hPalhNRFU4R0MzamI2S3NyTzlFRHV1UmprUlHSAaIBQVVfeXFMUERxLWVwMXlmWTRkQ3E3b2NUV0U1MFptMUhiR2FjMWMyOUlSbHM4NGl6NGc3ejI2TnI0R1ItNmt2U0UwUkZaU0xwWU43bjdkdmtJTXg1UTMwdUN6RXFubjhqNW1oZUxnWWJOZVNGRzZ2aHJ0Wmw5ekFBUHpYNDFaQWMxYUdfYy1uamptSmg4T0ZrYlZPdTNqdkNXU2N6U3I2OVN3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPRUtOa1hGa1ZkdTUxeUFQVFRKUGVPckRuNTZSVzRLUWdUSnZKS2lobVVNUXgzZEo2LUxFQ1B3X3FNa1dNcGdyRmNqX085N29XME1YTlpTR0ljakhOdm5janpYLVFaTkZKa2ZheE5qMWZyRnlhb1Y5VDQ0NUJUcGZOMXdBalZNbVBDMzBHNDJ0Ri1jVnAzZmtFMzl3dXNGQ3BSWFRua1p2eXhmbkVJNzJNWUdoSzhHTmNVRmgyQzhLUGpHdw?oc=5</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2234,7 +2234,7 @@
         </is>
       </c>
       <c r="K33" s="1" t="n">
-        <v>46121.87017361111</v>
+        <v>46122.06319444445</v>
       </c>
     </row>
     <row r="34">
@@ -2250,22 +2250,22 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>OPINION: Operation Budapest – Moscow Personnel in Brussels - Kyiv Post</t>
+          <t>VOLTAGE: Brussels wrestles with energy security concerns - Euractiv</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>OPINION: Operation Budapest – Moscow Personnel in Brussels - Kyiv Post</t>
+          <t>VOLTAGE: Brussels wrestles with energy security concerns - Euractiv</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 14:03:28 GMT</t>
+          <t>Fri, 10 Apr 2026 07:24:29 GMT</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTE1uTjF3UE9FQ0ZOYnRJeDVjR1doQ19kcWlCaFlta2dJT2RoQk1Kdnk1ZndEVVg4RTJ0NWs2QTZ0QVcxN1dEZTJUaDhxSHNJOGM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOTFp5UXBtTl9nWG5mZno4dVg1V2h2T0tPMEtpUlZxcDdESTRFeWVUUmczR1NJc0tfNlJUN0VXLXo1NkFFbzJoZkdHdkpQOTd5UUxkalV4U21Eb0RyT1k3VTY1VmhnclZlb3FlZV9mTTVfVXVaRjBFb1hGOGdYaVpYVGZEemZwNGNtbnJwN3JINA?oc=5</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2289,7 +2289,7 @@
         </is>
       </c>
       <c r="K34" s="1" t="n">
-        <v>46121.58574074074</v>
+        <v>46122.30866898148</v>
       </c>
     </row>
     <row r="35">
@@ -2305,22 +2305,22 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Belgian great Merckx set for surgery after hospitalisation - Reuters</t>
+          <t>International beer culture meets in Brussels - Brauwelt</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Belgian great Merckx set for surgery after hospitalisation - Reuters</t>
+          <t>International beer culture meets in Brussels - Brauwelt</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 15:53:43 GMT</t>
+          <t>Fri, 10 Apr 2026 01:19:14 GMT</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxPQzVEVGFQOVVoUVVFR0IwT3d0bjBaOTVCeHNWTTVFd3pmcTF4bU15RmpkQmlTSFVyRUJMcGg0WEUtUzMtbG1xQmVDZW84YmhaS1g1YzBkM0lDcTJieHR3bkpwaXhTcklMdUIySEFQc3d0UnNGRXQzY214M2xnaG13R0hXTENJQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOR3psMGtaUWhVak1vaXF0ejZSSWdTMVFsZF9kWERwTjBLY2dMUk9QVVl2dWJQVENBVWZpeVJuWmEtRk5ockotV1AtR3Zua1RESUFmXzgtTzBWS3owSTVNSHBGMGV5TmFpaGxzb1VWWVJnMUlUc01HLVR4aWtNa3Bha21EYTcyaGc4a0FHeWdKS200Q3JXamc?oc=5</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2344,7 +2344,7 @@
         </is>
       </c>
       <c r="K35" s="1" t="n">
-        <v>46121.66230324074</v>
+        <v>46122.05502314815</v>
       </c>
     </row>
     <row r="36">
@@ -2360,22 +2360,22 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Brussels backs windfall tax on big firms to ease pain from energy crisis - politico.eu</t>
+          <t>Israel, hands off the Christians of South Lebanon - Brussels Signal</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Brussels backs windfall tax on big firms to ease pain from energy crisis - politico.eu</t>
+          <t>Israel, hands off the Christians of South Lebanon - Brussels Signal</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 12:52:00 GMT</t>
+          <t>Fri, 10 Apr 2026 09:25:33 GMT</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQeVA0U1FYVHZHWEtYRFZkQ05sYjRsNmpCOGsyeDBhaGFVa0RnVS1JQy1wRjhfVkNkV2I2alU4S091Yjc1SVg0RF92MHFwUmhjanh0dVpVWHJpbXVzVHpHZVo3ZFBFX0c4VTh0VkxGWHdJWldMUnpkYVpfcVREMFp6QjVwNHFmT3pEeThaY3l1eGM2NTBsS2p3OWlfSlZ0UW8?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxOc09MeHJ3Mld6RGRDdnNSWTNYVU93WG1OLWhLcWRoS1J3eV9MNE0xbzEwSFBkZ1M3TndhcWs1N2ZGdDN2NkVxX0RrSEJSTlduNTZ5NUFnNjl1TXRhUXZtXzI0T2ZWOGNpNFBEekMwN3JvNVNEZERfdl8zaHVGNTFiYkhFWG5LWW1PSTE4?oc=5</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2399,7 +2399,7 @@
         </is>
       </c>
       <c r="K36" s="1" t="n">
-        <v>46121.53611111111</v>
+        <v>46122.39274305556</v>
       </c>
     </row>
     <row r="37">
@@ -2415,22 +2415,22 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>The Antwerp Six Were the "Myth That Kept on Living" - hypebeast.com</t>
+          <t>Artemis II: Countdown To Launch Day, Historic Mission Around The Moon Brussels (Es9X0AczRf) - Mshale</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>The Antwerp Six Were the "Myth That Kept on Living" - hypebeast.com</t>
+          <t>Artemis II: Countdown To Launch Day, Historic Mission Around The Moon Brussels (Es9X0AczRf) - Mshale</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 12:00:58 GMT</t>
+          <t>Thu, 09 Apr 2026 22:56:01 GMT</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE9fd1NoX04wcnBocFlqOTNNbUNCdEFSRVAxNGxiNzlkVzI0NWp1ZHZfMnhhMzEtb1Nldno2QzdLZnFRSkRGaTNPbGZxUFRVM1pWXzVlemRnbURRZFV3OVZXY1hTY3F1OHFuUnVyenBCM2Vhdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiY0FVX3lxTE83cjdOSFRTbjBXYjA5ZWxNNFY4YVhvdTBVOHlNOTNuZjJHdG1MbGJNcGNOVE14QnlfUDQ4ZkpXeGFESXh0dFlVRzI3WHhaVHFaVFlUcXEzam5wZEh5alM5Mk03RQ?oc=5</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2454,7 +2454,7 @@
         </is>
       </c>
       <c r="K37" s="1" t="n">
-        <v>46121.50067129629</v>
+        <v>46121.95556712963</v>
       </c>
     </row>
     <row r="38">
@@ -2470,22 +2470,22 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Thousands protest in Brussels against regional spending cuts - Anadolu Ajansı</t>
+          <t>Brussels finds humor amid online clamor - China Daily</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Thousands protest in Brussels against regional spending cuts - Anadolu Ajansı</t>
+          <t>Brussels finds humor amid online clamor - China Daily</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 15:44:05 GMT</t>
+          <t>Fri, 10 Apr 2026 01:15:00 GMT</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxPcXF1NDVGdmZkV2U5TnZSOEhxUDg2UXBYTnZaeXYybkxFUDJHVkFYaXcxLTVuajc0Yk1heVBUV3JLcFRua1NGWGNYTnJBSjZVdVBXajd3VE0yVzhsVG9yZk1HeVI1ZUh0WXFRSW51Z0VEaFpMX1FPZXY3SVo2TlpYZVpZYVVvS3ZyVUUzWjhDQUxLWnFlY0lCVWV4bw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1wSW0yYlR2MTUyXzNya3hWMlhfMHlVQWZQQzE0TTVROTRoQXJHcDUwVlZyb2M1VnBJN0R6VHdzQi0tSW50VHRZaWwzVko3ZW1pSVpEeWJxaW5sVlhFeHBJY2FnRWxqTmxyUl9TWmJmZDhwVmtDUU9icHhkb3hYQQ?oc=5</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="K38" s="1" t="n">
-        <v>46121.65561342592</v>
+        <v>46122.05208333334</v>
       </c>
     </row>
     <row r="39">
@@ -2525,22 +2525,22 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Kyrgyz Bank Wins Brussels Court Case Over Sanctions Accusations - The Times Of Central Asia</t>
+          <t>Resist or Submit: Hungary Votes on Brussels’ Grip on Power - The European Conservative</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Kyrgyz Bank Wins Brussels Court Case Over Sanctions Accusations - The Times Of Central Asia</t>
+          <t>Resist or Submit: Hungary Votes on Brussels’ Grip on Power - The European Conservative</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 12:44:46 GMT</t>
+          <t>Fri, 10 Apr 2026 10:27:45 GMT</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxQSWhqUmp4ZkhybjJaWGR6T1NJM0kzTlFOT2dNNHVXRWpla1FOaWtRTC1UMjRrMU9ENG9JVnpYWkxMMVhodEZabmpaSkRlTkViUG4zZFVudXppOU95UWt3cGpOQlBvM0lBMkdZV2FmVGxubmhUR1NrOGxkTGlscHVycDZrXzJ2MHdSSXlsaA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPTnBUQU8tZEpHMWg5Ry1RU0xEU2FEc3JpUkxFcHhfRWxSTzdMQ1RudEQ3RU5CZ3NPeHF5UUhNVEVhd0hPQ1ZuZ3VEdUxFa1ZZeWFPU2Q0QXV1VGpuQ3R4TXdtU2tRYjFiVEU0UmFYVzRZSHJlTTc4Q2MtOHBIRUIwM2RYdURHRGlVdE9IN1VHVlpoSk94R3JleEhteldGd1Q2cmxESkIwQQ?oc=5</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2564,7 +2564,7 @@
         </is>
       </c>
       <c r="K39" s="1" t="n">
-        <v>46121.53108796296</v>
+        <v>46122.4359375</v>
       </c>
     </row>
     <row r="40">
@@ -2580,22 +2580,22 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>The Mayor Gallery at TEFAF Maastricht 2026 - Artsy</t>
+          <t>Shanyraq Fest Brussels showcases Kazakh heritage in Belgium - Qazinform</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>The Mayor Gallery at TEFAF Maastricht 2026 - Artsy</t>
+          <t>Shanyraq Fest Brussels showcases Kazakh heritage in Belgium - Qazinform</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 18:31:13 GMT</t>
+          <t>Fri, 10 Apr 2026 03:58:57 GMT</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxNVjlaZ3JWZGw1MU0xaHR4dTJWS3JHMEtHTXRNRkZyMWNIX09UODVnNjkxWjlTZE1ScmpTMF9HYWlwZGduT1FtdkVCSTBMRDdsSG1oZWk0X2N6eGRWbFRZOEgyNmZoTVJFd24xOTc0ZDZHaTJDQXFHOHdPa1pIQmUydDJqcGV6ckRDRGxyVUotYl9FVW5iY3FR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQcUhzWjRISG1CYnV4ejc3elN6LUltZkUycUtBMTF1V0Z3SG9ibVo3Rm5STVRrZFBuZTdzRmtDbTBWV2ZMOUpsMGZnTGpSVDNsR2lrX0pjbUdlSlNyZW9oWFZJeVJvM0pPOVFBdHFaQUdFNDNTNHR0Z0VKdllrejdSc2FtT2tCQlZIcWNQZzE5SGNoVndfLU00YdIBmAFBVV95cUxQcUhzWjRISG1CYnV4ejc3elN6LUltZkUycUtBMTF1V0Z3SG9ibVo3Rm5STVRrZFBuZTdzRmtDbTBWV2ZMOUpsMGZnTGpSVDNsR2lrX0pjbUdlSlNyZW9oWFZJeVJvM0pPOVFBdHFaQUdFNDNTNHR0Z0VKdllrejdSc2FtT2tCQlZIcWNQZzE5SGNoVndfLU00YQ?oc=5</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2619,38 +2619,38 @@
         </is>
       </c>
       <c r="K40" s="1" t="n">
-        <v>46121.77167824074</v>
+        <v>46122.1659375</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>High Level City Belgium English (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Greece still has no justice for Giorgos Karaivaz as Brussels looks away - EUalive</t>
+          <t>Edito: stimuler l'utilisation du train, mais pas en deux minutes - Télésambre</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Greece still has no justice for Giorgos Karaivaz as Brussels looks away - EUalive</t>
+          <t>Editorial: stimulate the use of the train, but not in two minutes - Télésambre</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Fri, 10 Apr 2026 04:05:10 GMT</t>
+          <t>Fri, 10 Apr 2026 08:40:00 GMT</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxNNzRoRjhoV3hSSGdOS2phR1BpVWpid2xsMzBOUFRCQnkwZG5QVFh6TGZ3NGhTeDA4Z21KY3RFMkxDYllnb3JKMWhfZWh6ei1zM2RLbmNsekhrQmFybS1PcUg1b21nSmxPLVNicVN1TzFwR1RZWFNrTTdiSXZrMFI2eUJGZWt6YWV1cWhZYWVhTmt6YUQ4MU1Z?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNSFJKNHRIYnRUcmt3enMwczUxSW00NnMwOU5vTHg0ek5VckFmak5tdkNPcHhQVFVzSGF5cjREYUdERTdPZ1FfdGtfX3hKcUN5ekdmT3UzUklKa2tfSUotNnhFZ2pxeXp1RldWNHVYbEpzMkpWUm1FUkZWaEx0NG52d3NPTjVVMnVITXd2UU1IazFxVEkyVXkxTV96RjVmTTZR?oc=5</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2670,42 +2670,42 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K41" s="1" t="n">
-        <v>46122.17025462963</v>
+        <v>46122.36111111111</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>High Level City Belgium English (fallback)</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Our US poll expert in the heart of the campaign: ‘Hungarian election remains a tight battle’ - Brussels Signal</t>
+          <t>Chauffeur vervangbus NMBS tegengehouden in Hasselt met 0,2 promille in bloed | Foto - HLN</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Our US poll expert in the heart of the campaign: ‘Hungarian election remains a tight battle’ - Brussels Signal</t>
+          <t>Driver of replacement bus NMBS stopped in Hasselt with 0.2 permille in blood | Photo - HLN</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 10:06:21 GMT</t>
+          <t>Thu, 09 Apr 2026 17:35:02 GMT</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPUzFSLUFyaFRwaGhnYWhDTkx1bk9RSk9jamU4UFB4ZlNrNDVOaGU0Z012R0dfcTRrSUhJWlF5bVBLaHZNNnVHWXRHcFdPVE84bGE5cld5azlQc0RKbWptVDVKeGthN0NoWTBwbDJVNF9qN3ZteWdBdEtFU0JtdGJtX1RObEdNWmt6Ni1VY18wckgxUUZpNEVjQWNleWp0SDZ1TkV5RVY2V1pSYVIyb19oQlROSTdBRWpFelFVSnhuY2RFZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQWHhGalhhdERqSnNpNGp0cWVOeG9zMjYtT0h5UzZVT1RTTm9FT3F4M0VIdzl2Skg5cW44S0QtVXFXUDk4Qk5XVFRfX2NlSWtyQWo1WVB1SWFQdVRwQjloWDhMbFNCcTJIb2VhQXFkRU41dnZadkk0cGNpemVjOHQ2Z09hNC1hMHRDZWh3U0Y5Sm1TejNheFliWkJwRExLbjdQaW5ZT2J2c2NXeV9zUnFUdmEwcVpGSzV4WngxVWRVaFQ?oc=5</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2725,42 +2725,42 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K42" s="1" t="n">
-        <v>46121.42107638889</v>
+        <v>46121.73266203704</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>High Level City Belgium English (fallback)</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Orbán prepares to challenge Hungary election, critics warn - Contexte</t>
+          <t>Chauffeur van NMBS-vervangbus betrapt op alcohol in Hasselt: "Onmiddellijk ontslagen" - VRT</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Orbán prepares to challenge Hungary election, critics warn - Contexte</t>
+          <t>Driver of NMBS replacement bus caught with alcohol in Hasselt: "Immediately fired" - VRT</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Fri, 10 Apr 2026 06:00:00 GMT</t>
+          <t>Thu, 09 Apr 2026 14:30:40 GMT</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOLUo5OVdqQ0pEMWpCQ01YRldjU1hvYkhuZy1XUFdhZU1RaFR4QW1GdU5JWjJkMjY3SE1samZTSTZXRW40Y2ZLVDZvYWhndE44bzlzV3NwYWxuMkdtekhPc2VfZWRQbWo1QS0zRUhzVVVqQnZDOERIUGx6aENtamk5NzhQMXBXMWt3NWFUZ1hSb3pYTmNkOXhJcEd0aUFUZldpN3E4QUlOV2hwQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQcnRkUmtWQUFGaWJjU2x6ekNnUVQ4NnlBelFJN3djck84bEZqOHRyc3NGd2hkczkzeXplZFRNTEg0NldRTlVYTENYVkN2bEV4c2RNd1lxZ1VTSnlPTGdVY3BPRWthSjZyMHZIdTVHSEQtcm5vdnI2RFV1R0dMQmFlOFl3QzdGZVVZV3gzOUxKblBfWnhCMGRyTFFtU1NZMTlXclRqcG5OeVE?oc=5</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2770,7 +2770,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2780,42 +2780,42 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K43" s="1" t="n">
-        <v>46122.25</v>
+        <v>46121.60462962963</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>High Level City Belgium English (fallback)</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Huge rally at Brussels-Midi against cuts in French-speaking public sector - The Brussels Times</t>
+          <t>Terwijl het in de ene gemeente haast alcoholcontroles regent, blijft de teller in andere gemeenten heel laag staan. - HLN</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Huge rally at Brussels-Midi against cuts in French-speaking public sector - The Brussels Times</t>
+          <t>While alcohol checks are almost everywhere in one municipality, the counter remains very low in other municipalities. - HLN</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 21:22:30 GMT</t>
+          <t>Fri, 10 Apr 2026 04:27:13 GMT</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPaldSZk91Z3pXRGpKNmxURk1jU1J2c3RyWlRlM3RpLXVzN3lJQ1VOQmRlSmhhOUp3OEJmOEVmbm9mbnNKemxmeG56VmpubF81MHFQQVhOZXg3aGJuS2V3amFoTF9JOERUMDg1SXNJY19ZVU9mdmZ0Sm9mZUdKNWhna3BISmtPM1RBMmdSaVN2eDFQU3ZfYXJGTUdEOUwzbUU5T3UzS1VyN3ROQjN3TFpxLQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxOV01uT3pSUFNldS1QdS1PR1dxRk5EX2g0UHAwTWw4OWZfV0JYQjRtVjYtcmM5LTdlTHZfSEVnM20wa094N05OcEhPWlBZWEx6b2hSWW1xV1BqRjB6Z0pVYWtCN01DcGxsVjlNd29jdUJjN1RHTU45bjcwdWt2WDF2eWNtTDhIMmZHY1FoUTdJa1ozUEdTcjc4VElwSWdvMDRIZFVUWl9YdDlORUIwcHdKZDE0ZFk0emlENFdUYzR0eUo1VkVGSWJySXZ5TWw3eFk5bEU1Sk9OTW1xOW9rVUh5REJGczlyYVlkaG53Z3pBNA?oc=5</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2825,7 +2825,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2835,42 +2835,42 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K44" s="1" t="n">
-        <v>46121.890625</v>
+        <v>46122.18556712963</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>High Level City Belgium English (fallback)</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Belgium: E313/E34 motorway closed for nearly 6 days. Major disruption near Antwerp - trafficban.com</t>
+          <t>Grote verschillen in pakkans tussen gemeenten: zoveel alcoholcontroles deed de politie afgelopen jaar in Hasselt | Foto - HLN</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Belgium: E313/E34 motorway closed for nearly 6 days. Major disruption near Antwerp - trafficban.com</t>
+          <t>Major differences in the chance of being caught between municipalities: the police carried out so many alcohol checks in Hasselt last year | Photo - HLN</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 20:04:17 GMT</t>
+          <t>Thu, 09 Apr 2026 15:28:12 GMT</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTE96enVSQ2dJTU01LWpnZmpRVXBFUnR0Y3VuNy1BS1p5ZEpLU2dnbGZ2bUozekxQSkZ4dDVDOE1sejFVNVlxdW5yalRPX1NjR0hWMUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxNSkNTZ1gyVkdWNk1NdGZDemtMeXFFdnlEcUpXdDNyTmp3V2dPSUd3TjRpaXZRVndYWnN0SG9Mc052SWlwZzBFcm9sWThnemgxd1RlMjVWTGQxc0pNZUVmV2RjMVJyTlFLc2Y5d3c3Umt6N3JvMWd0cjUyaFNGSXNCM1poSkF0UWdObV9fdnQ3MWpDc3U4MWtBRF80YjRsZlY1aUp4OXRmRW85TlFoRlQ2Tjl4bXlkeUZZd2g1WVJOOWcwaUN4UHZIbTZ5SGMtU0E5MzVDdktRRHBPOUxWWG1VYnBkeHJFdDRhMWR3VTkxSQ?oc=5</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2880,7 +2880,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2890,42 +2890,42 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K45" s="1" t="n">
-        <v>46121.83630787037</v>
+        <v>46121.64458333333</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>High Level City Belgium English (fallback)</t>
+          <t>Local Town Maasmechelen English</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bomb OR explosion OR shooting OR stabbing OR evacuation OR police OR arrest OR threat) AND -sport AND -football</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Exclusive: Shell seeks to begin gas output at massive Venezuela-Trinidad Loran Manatee field next year - Reuters</t>
+          <t>Probability of alcohol check varies greatly by municipality in Belgium - The Brussels Times</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Exclusive: Shell seeks to begin gas output at massive Venezuela-Trinidad Loran Manatee field next year - Reuters</t>
+          <t>Probability of alcohol check varies greatly by municipality in Belgium - The Brussels Times</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 19:40:00 GMT</t>
+          <t>Fri, 10 Apr 2026 02:56:27 GMT</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxNQ01hczl3UXVISGhOWURFLVpvQndRUlBUY2RZaVR3dGRZcHBnaUtFaXFJd1NtNW9faUJIQjFkYnowNkFPaUkxTDlNUkFLaW1LOS05NGpMai0tWWt5RDBicFNZUWdlMEM5aTdRbHdKdWFaRzA2RzJheURSMVNTQ3YzaWU4RnIzeERhVE4zRm40SmpTVTQwbkdJZFJDc25aMkxyZjI4YUNxOFBETVJNYnBscDR2bjJhcVAwa29pZGthQkRuWFQ4RnZubzlhdHY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNNkdLajZFM0hzOEZzNDktMzBJa2JRSF9QYzJvb1k4ckoxY0wzUEZ6OTZLN19JLWdvNW05X21KYWtXaElQOHpQanpFalNtbldQRDRsWEN3OUJmQzB6Yzd3RFlMUTA5YUtRYU9reE9MVko1dXNXN3ZwXzFOUTV2WHlEOGJSUzBCNm9DeHZNVEhSdG9HRGs2UzloVEJOY0FvUEk1ZEgxWmJQMGpzN0pYa2NyQ0w0bnhfU2c?oc=5</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2940,47 +2940,47 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K46" s="1" t="n">
-        <v>46121.81944444445</v>
+        <v>46122.12253472222</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Maasmechelen English</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bomb OR explosion OR shooting OR stabbing OR evacuation OR police OR arrest OR threat) AND -sport AND -football</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Un train rapide entre Charleroi et Bruxelles dès décembre 2027 - Télésambre</t>
+          <t>E313 at Antwerp to close for five days, with major traffic implications - VRT</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>A fast train between Charleroi and Brussels from December 2027 - Télésambre</t>
+          <t>E313 at Antwerp to close for five days, with major traffic implications - VRT</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 08:00:00 GMT</t>
+          <t>Fri, 10 Apr 2026 08:17:24 GMT</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOZ1l3ZE1GcEdHSTBwMEtLeFZPWUNycmNSSl9uQ2RZWXNzc3ZxRmw5UHh3T2dIZC1kdlZiUWxOMGQwR2Y5ejhGczA0dlZ5YnI4dmV6TUdIZFRPR1U2aHk3eEtPUmNKcEFEM3lqZUZvb09Gbnhub3U2RV9CeXZxRFI4XzhjN0RhRk11bEtrallVX0RmcmEwaXpLUFVIRG8tTW8?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPeU1tOXVCcHZJaUQyY1JVNXFLSlhBSlRkb3JoYl9lckJPUEs4UmMwdzJyOFNMcFNBRk5Jck1EdUhNdDlmdFJzakhOa00wa0lURTU2QWx3MTdPdV9tdWpQSlJ6ZFJpZy1OampTMGJ4cjA3aTdPTHUzQVB2OGd2SEE2X2xZQ2U4c0t0TWNOUWUwQ0JCZEFQSDBVQkctX1lhUU5wNm1xNC1hZw?oc=5</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2990,52 +2990,52 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K47" s="1" t="n">
-        <v>46121.33333333334</v>
+        <v>46122.34541666666</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Village Wertheim (fallback)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Vidéos de menaces diffusées : un suspect interpellé et placé en observation psychiatrique - H24info</t>
+          <t>Suffolk County police rescue teen stuck in mud at Wertheim National Wildlife Refuge - AOL.com</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Threat videos broadcast: suspect arrested and placed under psychiatric observation - H24info</t>
+          <t>Suffolk County police rescue teen stuck in mud at Wertheim National Wildlife Refuge - AOL.com</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 08:00:47 GMT</t>
+          <t>Fri, 10 Apr 2026 02:29:55 GMT</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE83cjdNaGZGUTFTYjhDTVNjejJSOTFCZ25FYzRsYjRhQ251LWxkdzlYcDc4OVhpcm5vUkNjNkhodkphQ3JfMHRLcEp5NTdsSUpyQ0trbWtldDhlODFkTDRWNDJRT24yQU1VVzhpMmRDUzRnaUNCUHlzY1VB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTFB0dFQ0UUpCazdxSHBlS1djV0RFT1M0YWc5RHdmd3pRZnQtdS00OC1LcjVNUEY5dzAtdDE4TVZxaF9sbDFDN1NiT2hLQnIyWXVGNUhLbmRYRzRvWXc4djFrdk5Ebm8tMkE2RDRrQ1dDdVlRazlza0EwSkpra2g4UQ?oc=5</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3045,52 +3045,52 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K48" s="1" t="n">
-        <v>46121.33387731481</v>
+        <v>46122.10410879629</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Village Wertheim (fallback)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Chauffeur vervangbus NMBS tegengehouden in Hasselt met 0,2 promille in bloed | Foto - HLN</t>
+          <t>Yam Wertheim and Orly Yusupov • Two Against the Sea: The Israeli Journey to the Summit of the Aegean 600 - haipo.co.il</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Driver of replacement bus NMBS stopped in Hasselt with 0.2 permille in blood | Photo - HLN</t>
+          <t>Yam Wertheim and Orly Yusupov • Two Against the Sea: The Israeli Journey to the Summit of the Aegean 600 - haipo.co.il</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 17:35:02 GMT</t>
+          <t>Thu, 09 Apr 2026 16:11:37 GMT</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQWHhGalhhdERqSnNpNGp0cWVOeG9zMjYtT0h5UzZVT1RTTm9FT3F4M0VIdzl2Skg5cW44S0QtVXFXUDk4Qk5XVFRfX2NlSWtyQWo1WVB1SWFQdVRwQjloWDhMbFNCcTJIb2VhQXFkRU41dnZadkk0cGNpemVjOHQ2Z09hNC1hMHRDZWh3U0Y5Sm1TejNheFliWkJwRExLbjdQaW5ZT2J2c2NXeV9zUnFUdmEwcVpGSzV4WngxVWRVaFQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiSkFVX3lxTFBsdmNkRVFydlBjZVNWOGd2SWRNQUhGQkZKZHVvNkZmSm5fSlZBTGxLcW5mSW5JbXlsbGZDS1NxUzYwVkZDYTN0Zmp3?oc=5</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3100,52 +3100,52 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K49" s="1" t="n">
-        <v>46121.73266203704</v>
+        <v>46121.6747337963</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Village Wertheim (fallback)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Chauffeur van NMBS-vervangbus betrapt op alcohol in Hasselt: "Onmiddellijk ontslagen" - VRT</t>
+          <t>Helen and Jacob Shaham make landmark gift to FIU Medicine - Florida Hospital News and Healthcare Report</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Driver of NMBS replacement bus caught with alcohol in Hasselt: "Immediately fired" - VRT</t>
+          <t>Helen and Jacob Shaham make landmark gift to FIU Medicine - Florida Hospital News and Healthcare Report</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 14:30:40 GMT</t>
+          <t>Thu, 09 Apr 2026 11:41:28 GMT</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQcnRkUmtWQUFGaWJjU2x6ekNnUVQ4NnlBelFJN3djck84bEZqOHRyc3NGd2hkczkzeXplZFRNTEg0NldRTlVYTENYVkN2bEV4c2RNd1lxZ1VTSnlPTGdVY3BPRWthSjZyMHZIdTVHSEQtcm5vdnI2RFV1R0dMQmFlOFl3QzdGZVVZV3gzOUxKblBfWnhCMGRyTFFtU1NZMTlXclRqcG5OeVE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxOR0d6Qk1NSlRnS3JMQVlmR2c2WjFJX1B3WVpqSmx6QjJUcTdudkFHbXhSdnJWTHhFMUJQaE1idHgxc3ZHS0w5SzVuWUt2Wm8zWjZFem5UUzYxVXlnQnc4Mi1DNkJPZW1WZWRzNm4tRFFCdWxoZW9rM180cEwybU1Od2hFeGJGalVLbXJwQXVtZW5UeThhYkdLZXlJOA?oc=5</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3155,52 +3155,52 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K50" s="1" t="n">
-        <v>46121.60462962963</v>
+        <v>46121.48712962963</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Village Wertheim (fallback)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Terwijl het in de ene gemeente haast alcoholcontroles regent, blijft de teller in andere gemeenten heel laag staan. - HLN</t>
+          <t>Shirley Teen Stuck In Mud During Night Hike At Wildlife Refuge Rescued By Police Helicopter - AOL.com</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>While alcohol checks are almost everywhere in one municipality, the counter remains very low in other municipalities. - HLN</t>
+          <t>Shirley Teen Stuck In Mud During Night Hike At Wildlife Refuge Rescued By Police Helicopter - AOL.com</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Fri, 10 Apr 2026 04:27:13 GMT</t>
+          <t>Fri, 10 Apr 2026 02:43:07 GMT</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxOV01uT3pSUFNldS1QdS1PR1dxRk5EX2g0UHAwTWw4OWZfV0JYQjRtVjYtcmM5LTdlTHZfSEVnM20wa094N05OcEhPWlBZWEx6b2hSWW1xV1BqRjB6Z0pVYWtCN01DcGxsVjlNd29jdUJjN1RHTU45bjcwdWt2WDF2eWNtTDhIMmZHY1FoUTdJa1ozUEdTcjc4VElwSWdvMDRIZFVUWl9YdDlORUIwcHdKZDE0ZFk0emlENFdUYzR0eUo1VkVGSWJySXZ5TWw3eFk5bEU1Sk9OTW1xOW9rVUh5REJGczlyYVlkaG53Z3pBNA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE5kLVZfMmtON0RCVEI3ZEtfUmJhR2x2bC1BbFhYRVR1Nmxkb2M1UG1wdzIySjBzM3ktZWZmSm9RSFN1UEVzcHhvUHJhcEx5Z1dNN1JBMzNuTXdhbV9DNWdtOFFXdTJCQ2xMN2FPUjUtSnVNamRYdnhSTQ?oc=5</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3210,52 +3210,52 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K51" s="1" t="n">
-        <v>46122.18556712963</v>
+        <v>46122.11327546297</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Grote verschillen in pakkans tussen gemeenten: zoveel alcoholcontroles deed de politie afgelopen jaar in Hasselt | Foto - HLN</t>
+          <t>Ingolstadt: Vollstreckung Haftbefehl auf Autobahn 57 - Newsflash24</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Major differences in the chance of being caught between municipalities: the police carried out so many alcohol checks in Hasselt last year | Photo - HLN</t>
+          <t>Ingolstadt: Execution of arrest warrant on Autobahn 57 - Newsflash24</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 15:28:12 GMT</t>
+          <t>Fri, 10 Apr 2026 05:00:59 GMT</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxNSkNTZ1gyVkdWNk1NdGZDemtMeXFFdnlEcUpXdDNyTmp3V2dPSUd3TjRpaXZRVndYWnN0SG9Mc052SWlwZzBFcm9sWThnemgxd1RlMjVWTGQxc0pNZUVmV2RjMVJyTlFLc2Y5d3c3Umt6N3JvMWd0cjUyaFNGSXNCM1poSkF0UWdObV9fdnQ3MWpDc3U4MWtBRF80YjRsZlY1aUp4OXRmRW85TlFoRlQ2Tjl4bXlkeUZZd2g1WVJOOWcwaUN4UHZIbTZ5SGMtU0E5MzVDdktRRHBPOUxWWG1VYnBkeHJFdDRhMWR3VTkxSQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPa3BIUFM2Zk9vOW1nUUFFSS1KTW1KNHFhZ1JMc3F5ejFXTHZKMmpFM0RKaWJodHo0ZHppMDVNclFack1MMGlGOFg2a1poS2NIQllla3IxOHJqbDNtbjNWZGtRTk5vQnYzcDYxNTQ3NE1vRmQyenBaaWVTdDYxejFpM0Z3UnFaR0JzM0ltaVIxNmJTU0NucFRWTTFVMjRJSHFlTkRpLXZWQnc?oc=5</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3265,52 +3265,52 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K52" s="1" t="n">
-        <v>46121.64458333333</v>
+        <v>46122.20901620371</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French</t>
+          <t>Village Ingolstadt (fallback)</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Les perturbations restent importantes chez Bpost en Wallonie: celles en Flandre sont quasi terminées - 7sur7.be</t>
+          <t>Ingolstadt - top rated players, goals, assists and other stats - FotMob</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>The disruptions remain significant at Bpost in Wallonia: those in Flanders are almost over - 7sur7.be</t>
+          <t>Ingolstadt - top rated players, goals, assists and other stats - FotMob</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 08:45:00 GMT</t>
+          <t>Fri, 10 Apr 2026 01:45:22 GMT</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxOSk1EZ1owTnotc0NwdDBWWk15MzJ4dHFBeDFfQTBJbWI2R3VxSy1kNjdNMUI1LU80bWdkcldWMEFQNDJhbDNDMzVnWkd5eTNZQU8yU1JzcWRYN0RHaWVOMUhXcWNNMUtpMEdWNzVBQXpfaGpNbWxOaHYxOW5mbFhRc2hpN1NtVi1ZbXR3TnJqYlk1S3N5QmVBT1pzS3RGOEZxUDZwcVFyS0dmVUlybW9ZSW4xVDlGYzZQa0FXQVJJeUNTTGpRc1RpV09JQklhQTJ4aVFPTm53?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNLXhLNVVIWl9sOVNvUXNvUWNLZUpMX05DZmxDZ2JWejVnSldBY0NDRlJLUGlhWkMwOVBKRHRJUTVMVFhsQ3ZNbTg3Yy1BMG8xWHZNdS1jdThWQTEzUEFFdnYycEdQamlDWGdkQkt1OWdDMjRqMnQwVjhqcG5iWHZyUnRZUjYwa21Jc3hUSVdQZ2I4ZlBBYmU5OTRTMlF1MGpKU3QzaXhKQWZ0dXI5WVBmV3NB?oc=5</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3320,52 +3320,52 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K53" s="1" t="n">
-        <v>46121.36458333334</v>
+        <v>46122.0731712963</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English</t>
+          <t>Village Bicester Kildare</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bomb OR explosion OR shooting OR stabbing OR evacuation OR police OR arrest OR threat) AND -sport AND -football</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Probability of alcohol check varies greatly by municipality in Belgium - The Brussels Times</t>
+          <t>Entire Kildare on sale for €20 million - Newstalk</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Probability of alcohol check varies greatly by municipality in Belgium - The Brussels Times</t>
+          <t>Entire Kildare on sale for €20 million - Newstalk</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Fri, 10 Apr 2026 02:56:27 GMT</t>
+          <t>Thu, 09 Apr 2026 15:29:02 GMT</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNNkdLajZFM0hzOEZzNDktMzBJa2JRSF9QYzJvb1k4ckoxY0wzUEZ6OTZLN19JLWdvNW05X21KYWtXaElQOHpQanpFalNtbldQRDRsWEN3OUJmQzB6Yzd3RFlMUTA5YUtRYU9reE9MVko1dXNXN3ZwXzFOUTV2WHlEOGJSUzBCNm9DeHZNVEhSdG9HRGs2UzloVEJOY0FvUEk1ZEgxWmJQMGpzN0pYa2NyQ0w0bnhfU2c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxOT29OajNGWXNyY2JyWFk5X19WOXIxamhrYjJEc0RmaW1FLWFpQlFLanVPUWdzeXlFRmtuNnZSWVlVODZnM1l3TXc0aUtHLVF1bklGbWFVQ0RydGZxMWRkbGVQclNDVlBSajJJQmRVdU0yQWt4Sm83bVlwRXlnYWNuUklNZnZZQWxhRy1zUA?oc=5</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -3389,38 +3389,38 @@
         </is>
       </c>
       <c r="K54" s="1" t="n">
-        <v>46122.12253472222</v>
+        <v>46121.64516203704</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Village Wertheim (fallback)</t>
+          <t>High Level City UK Ireland</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" OR "Protest" OR "blockade" )</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Yam Wertheim and Orly Yusupov • Two Against the Sea: The Israeli Journey to the Summit of the Aegean 600 - haipo.co.il</t>
+          <t>Protester says they are willing to close Ireland down over fuel costs - BBC</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Yam Wertheim and Orly Yusupov • Two Against the Sea: The Israeli Journey to the Summit of the Aegean 600 - haipo.co.il</t>
+          <t>Protester says they are willing to close Ireland down over fuel costs - BBC</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 16:11:37 GMT</t>
+          <t>Fri, 10 Apr 2026 11:01:29 GMT</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiSkFVX3lxTFBsdmNkRVFydlBjZVNWOGd2SWRNQUhGQkZKZHVvNkZmSm5fSlZBTGxLcW5mSW5JbXlsbGZDS1NxUzYwVkZDYTN0Zmp3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE9jeHozYlNyM1czNkR4UHotZm9xUFRWM1ZoRWNqZXZTMTk4M3VoRnVpMmJXYzdWU0RjbTJmOGI5OHJhUm5veUNTcXNET2haTDkzVE1DSFdXX3NSUQ?oc=5</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3444,38 +3444,38 @@
         </is>
       </c>
       <c r="K55" s="1" t="n">
-        <v>46121.6747337963</v>
+        <v>46122.45936342593</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Village Wertheim (fallback)</t>
+          <t>High Level City UK Ireland</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" OR "Protest" OR "blockade" )</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Suffolk County police rescue teen stuck in mud at Wertheim National Wildlife Refuge - AOL.com</t>
+          <t>Primrose Hill stabbing witness urged to come forward with ‘vital’ video - ITVX</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Suffolk County police rescue teen stuck in mud at Wertheim National Wildlife Refuge - AOL.com</t>
+          <t>Primrose Hill stabbing witness urged to come forward with ‘vital’ video - ITVX</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Fri, 10 Apr 2026 02:29:55 GMT</t>
+          <t>Fri, 10 Apr 2026 08:59:32 GMT</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTFB0dFQ0UUpCazdxSHBlS1djV0RFT1M0YWc5RHdmd3pRZnQtdS00OC1LcjVNUEY5dzAtdDE4TVZxaF9sbDFDN1NiT2hLQnIyWXVGNUhLbmRYRzRvWXc4djFrdk5Ebm8tMkE2RDRrQ1dDdVlRazlza0EwSkpra2g4UQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNYV9WdFBNOGdWM0VsYUZ3SUlZeHh6N3BtbUdnRkZQOFBDSmt1eDlCVWNzV0ZhUVV3UFR4SU9RYlNvQmhpQkxSa1AxSmt3dU4yX0ZLM2EycVdOQkl6NXdYZmRqREVtSTVCcVFvaHdBVnk2eGZJdzRsZHlScF9ndlQxZXFvZjV5SGItWHN0bG9aeTFYMUlZMXAzNGthRV8tdVRZMVg3cURYWjhBRVRSUWdhR0dn?oc=5</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3499,38 +3499,38 @@
         </is>
       </c>
       <c r="K56" s="1" t="n">
-        <v>46122.10410879629</v>
+        <v>46122.37467592592</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Village Wertheim (fallback)</t>
+          <t>High Level City UK Ireland</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" OR "Protest" OR "blockade" )</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Helen and Jacob Shaham make landmark gift to FIU Medicine - Florida Hospital News and Healthcare Report</t>
+          <t>2026 film and high-end TV productions shooting in the UK and Ireland: latest updates - Screen Daily</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Helen and Jacob Shaham make landmark gift to FIU Medicine - Florida Hospital News and Healthcare Report</t>
+          <t>2026 film and high-end TV productions shooting in the UK and Ireland: latest updates - Screen Daily</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 11:41:28 GMT</t>
+          <t>Fri, 10 Apr 2026 04:00:26 GMT</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxOR0d6Qk1NSlRnS3JMQVlmR2c2WjFJX1B3WVpqSmx6QjJUcTdudkFHbXhSdnJWTHhFMUJQaE1idHgxc3ZHS0w5SzVuWUt2Wm8zWjZFem5UUzYxVXlnQnc4Mi1DNkJPZW1WZWRzNm4tRFFCdWxoZW9rM180cEwybU1Od2hFeGJGalVLbXJwQXVtZW5UeThhYkdLZXlJOA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQZmNMRTBhWHdsbFo0WHUtenBKUWJ0Z09LVVBuTjVUb1R6dnYyV0UwSEluX01NUXJuVzhuVlZCTUlHanpOQ0hpT1p4N2xGSnIyaEg3eGRKQ3BZVlJWT0hPREU4dmd2azc2VGVhQVl2emFKVmpENnNrT3BJNGVDY2xlNDVSUV95dzdPcHFtOHhqcG9WbUdYYU9odjhUTHp2b0dzMTZ6Yzh4U1VGNVVfeVl5RmQ1eDJpLU91MHlMUS1kZlZNNng3LTE1VHNIb1o?oc=5</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3554,38 +3554,38 @@
         </is>
       </c>
       <c r="K57" s="1" t="n">
-        <v>46121.48712962963</v>
+        <v>46122.1669675926</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Village Wertheim (fallback)</t>
+          <t>High Level City UK Ireland</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" OR "Protest" OR "blockade" )</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Shirley Teen Stuck In Mud During Night Hike At Wildlife Refuge Rescued By Police Helicopter - AOL.com</t>
+          <t>People walk with luggage past heavy traffic on Dublin's M50 - BBC</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Shirley Teen Stuck In Mud During Night Hike At Wildlife Refuge Rescued By Police Helicopter - AOL.com</t>
+          <t>People walk with luggage past heavy traffic on Dublin's M50 - BBC</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Fri, 10 Apr 2026 02:43:07 GMT</t>
+          <t>Thu, 09 Apr 2026 21:44:45 GMT</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE5kLVZfMmtON0RCVEI3ZEtfUmJhR2x2bC1BbFhYRVR1Nmxkb2M1UG1wdzIySjBzM3ktZWZmSm9RSFN1UEVzcHhvUHJhcEx5Z1dNN1JBMzNuTXdhbV9DNWdtOFFXdTJCQ2xMN2FPUjUtSnVNamRYdnhSTQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFBlV3lxS3VZRHYtY1hESzNJSWJ1OElRRzA1ZXdmUHdTVU5BQVVTczVveWpDNGpDcWhuanBrY28xS21ic0ozUk5OZFhPbEhrYjdZSjN3U0xSVml2Zw?oc=5</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -3609,38 +3609,38 @@
         </is>
       </c>
       <c r="K58" s="1" t="n">
-        <v>46122.11327546297</v>
+        <v>46121.90607638889</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City UK Ireland</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" OR "Protest" OR "blockade" )</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>65-jähriger Rennradler stürzt bei Kösching und verliert das Bewusstsein - Pfaffenhofen Today</t>
+          <t>Live: Martin's Canada trade mission postponed amid protests - RTE.ie</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>65-year-old racing cyclist falls near Kösching and loses consciousness - Pfaffenhofen Today</t>
+          <t>Live: Martin's Canada trade mission postponed amid protests - RTE.ie</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 11:33:11 GMT</t>
+          <t>Fri, 10 Apr 2026 05:18:33 GMT</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiY0FVX3lxTE1QR0xiUHlUT05WTVRPV1pzQXJ4V05QRGNUemF5d1A5T2NZeWdaMVhqbmRISnJwdkdESXRhZ3VIcWp2LVRJT01pR3FCZHhwZkJLd0IxMnZVVF9ubHhKeDFRMnViVQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE9FVHJpN1liQXd2cEwzVklEWFV3UklZNUxvT0pQSFZ1c2xzcW1peGZQZ2tOV2UtQ0NJbmwzYVVkcWEwUTh3UTNzRXJLcHc5REtTYXRtU3cyb1RCQVp0OHVVOFhVeEtRX0U?oc=5</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3650,52 +3650,52 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K59" s="1" t="n">
-        <v>46121.48137731481</v>
+        <v>46122.22121527778</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Village Ingolstadt (fallback)</t>
+          <t>High Level City UK Ireland</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" OR "Protest" OR "blockade" )</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Ingolstadt - top rated players, goals, assists and other stats - FotMob</t>
+          <t>Primrose Hill stab victim 'can never be replaced' - BBC</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Ingolstadt - top rated players, goals, assists and other stats - FotMob</t>
+          <t>Primrose Hill stab victim 'can never be replaced' - BBC</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Fri, 10 Apr 2026 01:45:22 GMT</t>
+          <t>Thu, 09 Apr 2026 18:10:50 GMT</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNLXhLNVVIWl9sOVNvUXNvUWNLZUpMX05DZmxDZ2JWejVnSldBY0NDRlJLUGlhWkMwOVBKRHRJUTVMVFhsQ3ZNbTg3Yy1BMG8xWHZNdS1jdThWQTEzUEFFdnYycEdQamlDWGdkQkt1OWdDMjRqMnQwVjhqcG5iWHZyUnRZUjYwa21Jc3hUSVdQZ2I4ZlBBYmU5OTRTMlF1MGpKU3QzaXhKQWZ0dXI5WVBmV3NB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE9MQlc0SWFhUXljdmFhaXp2QmFyUHBScTI5MlVReDdienR6cUloUm1FLVpReGo1MW9nU1FDVFBGSFY4R3NIZGFEekFzODAzWDM0czhVU3NOOUpWdw?oc=5</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3719,38 +3719,38 @@
         </is>
       </c>
       <c r="K60" s="1" t="n">
-        <v>46122.0731712963</v>
+        <v>46121.75752314815</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare</t>
+          <t>High Level City UK Ireland</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" OR "Protest" OR "blockade" )</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Entire Kildare on sale for €20 million - Newstalk</t>
+          <t>Irish army called in to remove fuel depot blockades - Sky News</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Entire Kildare on sale for €20 million - Newstalk</t>
+          <t>Irish army called in to remove fuel depot blockades - Sky News</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 15:29:02 GMT</t>
+          <t>Thu, 09 Apr 2026 13:27:24 GMT</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxOT29OajNGWXNyY2JyWFk5X19WOXIxamhrYjJEc0RmaW1FLWFpQlFLanVPUWdzeXlFRmtuNnZSWVlVODZnM1l3TXc0aUtHLVF1bklGbWFVQ0RydGZxMWRkbGVQclNDVlBSajJJQmRVdU0yQWt4Sm83bVlwRXlnYWNuUklNZnZZQWxhRy1zUA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxQSXg5a3JKaTY3c0FGQnBpOUJRY0lQVC1tYVZaMnNKU2hnS3dhaUhGZjNWVFpGanpwdHRiU2FqR3FwdWQtNzJYSkpoSFNTMDdmNkxqZ05VMnNaLUtPdnhUZWpBenZyT2FUVTNQUnNSako4Y3ptbkxlM3NvcXJocUR5QlNpMVFWR05WeGFVSkt3VFE?oc=5</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3774,38 +3774,38 @@
         </is>
       </c>
       <c r="K61" s="1" t="n">
-        <v>46121.64516203704</v>
+        <v>46121.56069444444</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare</t>
+          <t>High Level City UK Ireland</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" OR "Protest" OR "blockade" )</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>KASH Beauty’s 90s Collection Is Here – &amp; We’re Obsessed - stellar.ie</t>
+          <t>Tate Modern evacuated and Millennium Bridge closed in police incident - London Evening Standard</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>KASH Beauty’s 90s Collection Is Here – &amp; We’re Obsessed - stellar.ie</t>
+          <t>Tate Modern evacuated and Millennium Bridge closed in police incident - London Evening Standard</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 11:01:04 GMT</t>
+          <t>Fri, 10 Apr 2026 11:13:11 GMT</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPZDZLUURBbHA5NmRwbVBIVHNLQy1fZkFzOWd4QTdyRGc0RU41RFNMeThrSnVOOGRwNXhvYkd3VHpRMjdKdVh2aHE3THBtZGM3NDk1MjVlNlJVb3puM1pGa0UzOG8tZ0J2N2p1UXdiV0hkcEc5elFOc1JiSHBNUG92Z2tvZUEzbUhLNlg5ZWdmckliQ2ts?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOVXAzUGp1TndFUXlXMDJHVnJBcU8tU0FrcnFqc3htcElkWE5pVUJ6V25LZmJDSEY3M1pYTXJJZGtiT1M1UlNyb1R3SHk3X0pHMEZ6MFZkSVphSHpuTkJhUG1JTVVuUEhHQm02NWdhTnhZOHMtV2ZBNUxJSGRtZnBfWGZqUERjWUhEMDFTQk0xZEgxeW1OLU1DaUx5OFN6a1BONU1yT0FVTHEwaS1aRDc2Wk5EY0E?oc=5</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3829,7 +3829,7 @@
         </is>
       </c>
       <c r="K62" s="1" t="n">
-        <v>46121.45907407408</v>
+        <v>46122.46748842593</v>
       </c>
     </row>
     <row r="63">
@@ -3840,27 +3840,27 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" OR "Protest" OR "blockade" )</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2026 film and high-end TV productions shooting in the UK and Ireland: latest updates - Screen Daily</t>
+          <t>‘Panic buying’ setting in on fourth day of fuel protest - East London Advertiser</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>2026 film and high-end TV productions shooting in the UK and Ireland: latest updates - Screen Daily</t>
+          <t>‘Panic buying’ setting in on fourth day of fuel protest - East London Advertiser</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Fri, 10 Apr 2026 04:00:26 GMT</t>
+          <t>Fri, 10 Apr 2026 01:54:27 GMT</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQZmNMRTBhWHdsbFo0WHUtenBKUWJ0Z09LVVBuTjVUb1R6dnYyV0UwSEluX01NUXJuVzhuVlZCTUlHanpOQ0hpT1p4N2xGSnIyaEg3eGRKQ3BZVlJWT0hPREU4dmd2azc2VGVhQVl2emFKVmpENnNrT3BJNGVDY2xlNDVSUV95dzdPcHFtOHhqcG9WbUdYYU9odjhUTHp2b0dzMTZ6Yzh4U1VGNVVfeVl5RmQ1eDJpLU91MHlMUS1kZlZNNng3LTE1VHNIb1o?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQdC1xdDA2SGJwYnZ1c29fT0R4QnVRSnlUU09YMzVMbnBYRjZqWXdkVnhvWHdCYkVGY0pfXzJyYWNKS25ieTN0MkVVU1BoZVR3eTF1WEtnWGlsdVJVMS1sVkEweWpYN3RFOTRjVmVaYjNSX1FMQmFWMHpwRGF3Z0dDdmZYeGNRZWYwdVdNbFRYT1QtQy1kT0poNEtxb3RCY1VNeXdEdi1kYWd5SUE?oc=5</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3884,38 +3884,38 @@
         </is>
       </c>
       <c r="K63" s="1" t="n">
-        <v>46122.1669675926</v>
+        <v>46122.07947916666</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>High Level City UK Ireland</t>
+          <t>Village La Vallee</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("La Vallee Village" OR "LaValleeVillage" OR "LaValleeVillage" OR "Ingolstadt Village" OR "IngolstadtVillage" OR "IngolstadtVillage")</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Student killed in Primrose Hill stabbing named by police | ITV News - ITVX</t>
+          <t>La Vallée Village Joins the European Artistic Crafts Week - Luxus Plus</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Student killed in Primrose Hill stabbing named by police | ITV News - ITVX</t>
+          <t>La Vallée Village Joins the European Artistic Crafts Week - Luxus Plus</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 11:37:00 GMT</t>
+          <t>Fri, 10 Apr 2026 05:54:54 GMT</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxOVDR1eXNVSkszQ2pHcXlmcXhHSWdvTnZ2N2JaTUE1cHFDcGdhMDdsWEFlOGY3allfczhvbFBNbVFPekJDRVFVbmtUdjVmUDhzZElzR3ZQN0llRFdPOEI1RjN6cXpTX3h5QlRiTlBkN28wYlhhaklwZFB5MHo2OC1nNG5ZbXJtTXhfRXRwWkk1dDd4UDZq?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNVVVDbWEzRGVEZlZFZmE1b2hFdVAtVW1nVHY2RXFLbmxISmkyUkZsOU9OeXZLSWhMaGlydGY5MVBNNWlMdzAzN2VLTWRoU0hwTEJzU3JWbkw3WThIVnFCbkIyV1ZfUUN4T19zRHlsT3lPUnRWbDU0YVZxTnlQNWFLekZSTm1CQmNvS0RoVQ?oc=5</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3939,38 +3939,38 @@
         </is>
       </c>
       <c r="K64" s="1" t="n">
-        <v>46121.48402777778</v>
+        <v>46122.24645833333</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>High Level City UK Ireland</t>
+          <t>High Level City Italy English</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Milan" OR "Milano" OR "Bologna") AND ("Italy" OR "Italian") AND (protest OR demonstration OR rally OR "civil unrest" OR strike OR blockade OR march) AND -football AND -transfer AND -Serie AND -"fashion week" AND -catwalk AND -runway</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Primrose Hill stab victim 'can never be replaced' - BBC</t>
+          <t>Italian Air Traffic Controllers Set for 4-Hour National Strike on 10 April—Hundreds of Flights Already Cancelled - VisaHQ</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Primrose Hill stab victim 'can never be replaced' - BBC</t>
+          <t>Italian Air Traffic Controllers Set for 4-Hour National Strike on 10 April—Hundreds of Flights Already Cancelled - VisaHQ</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 18:10:50 GMT</t>
+          <t>Thu, 09 Apr 2026 22:09:14 GMT</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE9MQlc0SWFhUXljdmFhaXp2QmFyUHBScTI5MlVReDdienR6cUloUm1FLVpReGo1MW9nU1FDVFBGSFY4R3NIZGFEekFzODAzWDM0czhVU3NOOUpWdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxNTEZyb0gwVjI0V1FaTjg4VXluWV82aWJfa1dLUk1UdmE1b0xDR1J5ZTNmdzFyaENQMm1Lc3dCSWVEbnhIYi1NdHMwQldYbGhPQ1dpNnBtOTdRX1U3N2RlM1F6dkNCUWdYVWQzeTRnV1hxS191OHkwUjBuTzFRa0w0ZDNXb29NTzZva3hVcTh1WHVDSWNvQ3VkYUo1S1BqY0xLcURULWszd3hpbEtET2VlRTBZQjV6M01xY1F2dkdQOTY3eHdaT0tUSENJSW1ISTFwWmdmeG9EMzZlRnEzOEQ0b29ZZ0MzRTFQZEVR?oc=5</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3985,47 +3985,47 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:en</t>
         </is>
       </c>
       <c r="K65" s="1" t="n">
-        <v>46121.75752314815</v>
+        <v>46121.9230787037</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>High Level City UK Ireland</t>
+          <t>High Level City Italy English</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Milan" OR "Milano" OR "Bologna") AND ("Italy" OR "Italian") AND (protest OR demonstration OR rally OR "civil unrest" OR strike OR blockade OR march) AND -football AND -transfer AND -Serie AND -"fashion week" AND -catwalk AND -runway</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Small boat migrant with unknown age imprisoned for Oxford university stabbing - Oxford Mail</t>
+          <t>Strikes by Italian air traffic controllers and Lufthansa staff affect Luxembourg flights - Luxembourg Times</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Small boat migrant with unknown age imprisoned for Oxford university stabbing - Oxford Mail</t>
+          <t>Strikes by Italian air traffic controllers and Lufthansa staff affect Luxembourg flights - Luxembourg Times</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 11:15:00 GMT</t>
+          <t>Fri, 10 Apr 2026 08:05:53 GMT</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOaHFBWTRUWXZOTU1zc2laejFxbmNvdjFxTjFaYy00STV1MWNoNGROTDVrOWlFSDJhaXE2aUxMOGRnZzhJb25QV1M5R2NOQ2dLVEx6N284QWVXOGllTWFtVGpLUXRldzB5T1lmUkxvQ1pUbzFOYVhyUHFDa0t6Q2h1cmhkVDNBd013bVRLOHR0LTc5V3pSTXl4cnhjdzhIZDAtVUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxNamdpZHF4cW92ZFUyMVdra25KYVJ3UjRCU1Q1VWRhOWFPbmdBd0hmSzRFZ2ZOTzJxazRlNTVjSE4wZ25wRXl0QmVNdFh3N0FzcDJnMjM4Z1FGOVcyYVU0M1hJVUExdnRya2Z2cXFEU3ZJY1JmUDJPZy15TjNBbk10YTlBdGUwM1NjNmJuQU9sSTEwMm5HN0Z5UTlXcWdIeklWMno4cmx3Q2lZcDVrYnJmR1AzdmhHZFNrWmhpWEhJYUxKOFdDV2FoYmVYTlJHaFhKVDJPcQ?oc=5</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -4040,47 +4040,47 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:en</t>
         </is>
       </c>
       <c r="K66" s="1" t="n">
-        <v>46121.46875</v>
+        <v>46122.33741898148</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>High Level City UK Ireland</t>
+          <t>High Level City Italy English</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Milan" OR "Milano" OR "Bologna") AND ("Italy" OR "Italian") AND (protest OR demonstration OR rally OR "civil unrest" OR strike OR blockade OR march) AND -football AND -transfer AND -Serie AND -"fashion week" AND -catwalk AND -runway</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>‘I’m broken-hearted’: father pays tribute to student, 21, stabbed in Primrose Hill - The Guardian</t>
+          <t>FTSE MIB Today: Milan Edges Lower as Italy's Blue-Chips Consolidate Ceasefire Rally - BBN Times</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>‘I’m broken-hearted’: father pays tribute to student, 21, stabbed in Primrose Hill - The Guardian</t>
+          <t>FTSE MIB Today: Milan Edges Lower as Italy's Blue-Chips Consolidate Ceasefire Rally - BBN Times</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 08:31:00 GMT</t>
+          <t>Thu, 09 Apr 2026 20:04:24 GMT</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNUk5RN2NXX2M4WTVnZEJuamFRNWJvTng0SnlNWlZjZTMyMDFoN01jRlNOaDRyMlRJYV93NVZsUDlBUnFOaDRuZW1ndl9GdUxzZEhfQ3lSX3ByZ09PWGhiOWRSZXlzaGY4UHFQdnBtTlVCWFpSSEZtOGpkS0ViaEJDMDFBcjRCWTZGeURtbEVwaHVxazlsMXVmWTR2YnhFQlhqREplbFNPcUh5ZHFiWlVqNGYtM1NKZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxNM0V0TzBvQm9SWlFTV1VONldxVjN0bzRqYjlIRzZRRDlzeEQ3OVdTTWt5c3AwVE4yUVQ3T1ZfeFB4UUhqbHpuc0lTRDlodW01MHVSZEFhN1dlZHJJaGNYRmg3eWdza1FjLTc5M0xQV21YMVpEOFBwU3pKMVdnb3pNeWFoRmhjLWlwQndiRWw0aEtIZUIzRXJ1OFBQUTFMMV85OUM0c1pwUkd0U2RTTjJfR3RkamlFV3JYdkNRb0xBSlFLTi05WkJMNy01djB6Zw?oc=5</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -4095,47 +4095,47 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:en</t>
         </is>
       </c>
       <c r="K67" s="1" t="n">
-        <v>46121.35486111111</v>
+        <v>46121.83638888889</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>High Level City UK Ireland</t>
+          <t>High Level City Italy English</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Milan" OR "Milano" OR "Bologna") AND ("Italy" OR "Italian") AND (protest OR demonstration OR rally OR "civil unrest" OR strike OR blockade OR march) AND -football AND -transfer AND -Serie AND -"fashion week" AND -catwalk AND -runway</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Friend heard 'screams' in last phone call with Primrose Hill stabbing victim - London Now</t>
+          <t>Due to nationwide strike: Air traffic between Luxembourg and Italy disrupted on Friday - RTL Today</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Friend heard 'screams' in last phone call with Primrose Hill stabbing victim - London Now</t>
+          <t>Due to nationwide strike: Air traffic between Luxembourg and Italy disrupted on Friday - RTL Today</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 16:08:35 GMT</t>
+          <t>Fri, 10 Apr 2026 05:41:07 GMT</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNR0I0NExPRkFDTkZaZFdDNDdKOGUzY0pzeUdfY1NzRGQ4dDRELUIzU0xnWW5ROGhkTE50Ny0xWi1NQ3lSRjdSbDdpRGVEUGhtNk5LOTRtbDBISnFoZTdsRjEtclpzU1E0MHI2NDJLclE3WTAxODhPU2hsSGdxMDFZeVRBTTdEdFNmY0tkaWdEUzdTb3A3TWJXd3BPUFNnZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQdGl2SWlUblZQWXhORkE0Y1lZRmZaRkljeHBZOHlYLXVWUjExOTFSS1JwWl81d29OcU1hOXZZaE1QUm9GX3dDb0JLOEZ6V2RYVjVOUUhwbjRFMDF0bjBtTW5SLWNlTGROT2hBRVdOby1iOTc4dWlHb3ItVG9lWDdFbkc4TmRWdzhqVlRSNTFSRTBON3VKMjVYdFh6YWJDS012RjdDSmRHLWdrd0k?oc=5</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -4150,47 +4150,47 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:en</t>
         </is>
       </c>
       <c r="K68" s="1" t="n">
-        <v>46121.67262731482</v>
+        <v>46122.23688657407</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>High Level City UK Ireland</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Boy, 17, rushed to hospital after shooting in south east London - London Now</t>
+          <t>Lunedì consiglio federale Lega a Milano, fari sulla "manifestazione dei Patrioti" - il Nord Est</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Boy, 17, rushed to hospital after shooting in south east London - London Now</t>
+          <t>Lega federal council in Milan on Monday, spotlight on the "Patriots demonstration" - the North East</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 13:50:46 GMT</t>
+          <t>Fri, 10 Apr 2026 09:14:04 GMT</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxQZ0k4ck44WmRkb25fZzdtUjFvZ0cwWlA5WmR1NDB1Ri1DV3JUbEY5eWZ3MWtlQWdJNG1OeTVTTU8wdkZlN3JraThQZm45eVZuQTUzakw0S2xTSVdEbGl3VGZCX1FXejRpajJIa00tQUlURmNaUU83RVM3ZWgwbE5qc3VKT1E5SW5TT0szMFpsREMtbEZMM1JmZWMza3pBdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxNNXBBTXNLWHVtOXNzcWNMa1FmS3ZsMXNpb3FNTVFEV1VNX2QzNFYzSFBhTFlEOTJ2MW9xVjJleEttaE5rQlVwc0VwUjNROGxwLUZadWJsSGJxY0tTV2RkY1haMUJEYnd0N1pFbk40WW90TnFQcHM2SGZjc0NVQWxIbzB6VmplZWp4U25CRWRfQjVnd0tHenFrcE44eldGVTA2OWhsLXNJczF3RzNtYTVHUkJEQmpvelJRYng4X2FmQjV4Ukt1enU5Tw?oc=5</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -4200,52 +4200,52 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K69" s="1" t="n">
-        <v>46121.5769212963</v>
+        <v>46122.38476851852</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>High Level City UK Ireland</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Man stabbed to death ‘seen falling to the floor in front of crowds’ near busy market - London Now</t>
+          <t>Milano. Lunedi processo a sindacalisti e studenti per la manifestazione sotto Assolombarda - Contropiano</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Man stabbed to death ‘seen falling to the floor in front of crowds’ near busy market - London Now</t>
+          <t>Milan. Monday trial of trade unionists and students for the demonstration under Assolombarda - Contropiano</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 11:17:55 GMT</t>
+          <t>Fri, 10 Apr 2026 09:48:54 GMT</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxObFE2RkhmQkN4VEl1SWZ5TDNJOVdoSURjN2p2UXpMeVU0X3Y3Q0dGLXlaUlJCX1c5YkFyZl80cjNzLXlQUVlpZlAtTmdELVhxZ19IMnFRSWZxaDY0cFUtYlNrMXZqSlZSMHozanhFeExqUU93UVZDSENZM015Ym8yYkxIcmdIOTNhUkRyanRJRWthOTQ3c0Q0M2FQOEdwS25OYVBJ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxOTFJtb3pnM0tpSzdTejA3TnVVXzVTWm95eFg3UTJTX0pob3FOaDdyczc2WXpOVkxJVDlMUjRjQkZZMWE1c2gwQ0pQOEYtbnc1eXU2NVh3LU5mR2JwZmEwblhtN1N6VUZNNi1FQ0I0TXdVUVMtbDJGUUVDOV9OVHRBb2JacDlQczVDZE9nMU8ycmlzdnVRbkFGb2t5SEFKYUpSUE4zcFpNNU0xM1h1RXJHZ0Jycy03dzN1QkloTEhPdUFuUm1DTmxhLXlrd3JzaXNtaTdpYkY2QWRiSHd3aVhac2FQV3hsZFVPSEtQN3RwMVg?oc=5</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -4255,52 +4255,52 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K70" s="1" t="n">
-        <v>46121.47077546296</v>
+        <v>46122.40895833333</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>High Level City UK Ireland</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Shrine for father’s only son stabbed to death at London viewpoint - London Now</t>
+          <t>Nuovo sciopero dei treni l'11 aprile: viaggi a rischio nel week end - NovaraToday</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Shrine for father’s only son stabbed to death at London viewpoint - London Now</t>
+          <t>New train strike on April 11th: travel at risk over the weekend - NovaraToday</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 12:00:12 GMT</t>
+          <t>Thu, 09 Apr 2026 12:54:47 GMT</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxQbUxfWG12dlNBdklVUzVvT0hTVGNvYkhvbG5wZ3FSUTA3RDNETW43bnhQS01BOGxEV1JteEo3VmNVZDM4VkN6MWF6YktlVUVfRWdELW5reFdqVmpjYXdmRHlLdXRDZjNnUGZTanFEMElTd1RQRWppRmZvYzJXRlJqMS1SSkdYbkdNYjlESFNkU01QVTRqdjh5U2JkNzlhdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE95NXFTMks5ODJoSjNsMlZqZW1vVl85dllZRW1NYTlvRDVMYnJsWU1NUklQV3ZPMXp3XzUwT19OMHR5NUxXRnd2UTlqUHJhc3I0QndWZ3E2MmxYNXlON3BaZFJpaTZRWU5Wbm1hWHFwYjFjNjBzRDViNnhIMA?oc=5</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -4310,52 +4310,52 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K71" s="1" t="n">
-        <v>46121.50013888889</v>
+        <v>46121.53804398148</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>High Level City UK Ireland</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Tate Modern London Evacuated After Bomb Scare - National Today</t>
+          <t>Milano: Lega protesta contro no a Remigration summit, ”stop Fascismo rosso” - Foto - Agenzia Nova</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Tate Modern London Evacuated After Bomb Scare - National Today</t>
+          <t>Milan: Lega protests against no to Remigration summit, "stop red Fascism" - Photo - Agenzia Nova</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Fri, 10 Apr 2026 06:46:57 GMT</t>
+          <t>Fri, 10 Apr 2026 05:19:40 GMT</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQQjl3RFJnaVAtM19WZVBaWGRhZkV2N19SREloRGpONnhaQVBxTkx0QmoybElPR0d5TVM2QVhGTjRxeml3Ui1LanhWaW1tcS10alZMOFRXazEyX25lUmh5S3lqV2RtRjJuckdvTkVGX2pEbnZMZkxWSjI4STZaUHBqVkNKeXNvOFBDMU9WYlVhQzVNZUpsRTcwX0VtSmdVZlR5R3c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxPS3Ywak5RZ3d3bnVxVnFURFNqRGZvQTEzZ2R0QU1YdlU3UTF4bWYyT2NPbDQ2MVhBOEFrT0k4VVItSEhBQVhiS0YxbGkzX2lJenhGNGw1MkgtdEZBSDNHeHVNbDE2Wlg2aURjZG1LZzVqcHJ0V3lhdm9iZnNrSEVRVkRHb2tzTkhGQ2FUN09qdVYzSm5OdGxvMHpUbVRJNzB5NEZHTHBQSXdsbjV4UWo4X3BlRnMzTEZwTHM2bnpRTUpiRjJ3b3N6ekFIWTFmaFFNMGk3ZUhJbTVqNkZ0NlBSc0NjTQ?oc=5</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -4365,52 +4365,52 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K72" s="1" t="n">
-        <v>46122.28260416666</v>
+        <v>46122.22199074074</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>High Level City UK Ireland</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Tate Modern evacuated and Millennium Bridge closed in police incident - London Evening Standard</t>
+          <t>Dopo Pasqua arriva lo sciopero degli aerei - Moveo by Telepass</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Tate Modern evacuated and Millennium Bridge closed in police incident - London Evening Standard</t>
+          <t>The airline strike arrives after Easter - Moveo by Telepass</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 13:03:00 GMT</t>
+          <t>Fri, 10 Apr 2026 06:21:42 GMT</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOVXAzUGp1TndFUXlXMDJHVnJBcU8tU0FrcnFqc3htcElkWE5pVUJ6V25LZmJDSEY3M1pYTXJJZGtiT1M1UlNyb1R3SHk3X0pHMEZ6MFZkSVphSHpuTkJhUG1JTVVuUEhHQm02NWdhTnhZOHMtV2ZBNUxJSGRtZnBfWGZqUERjWUhEMDFTQk0xZEgxeW1OLU1DaUx5OFN6a1BONU1yT0FVTHEwaS1aRDc2Wk5EY0E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiaEFVX3lxTE54azFfZG9yU2RiMVlFTDFNSU55V09oRGxJZzY0cGVjSWVZVXhsbXFfZlhvWTZ1VHktZ2h1RFJleUFDM2FHbWxyeE4xYnBCcWd2MXpKOFFDdU1mci13NG1QaDBxZ2FjYnBk?oc=5</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -4420,52 +4420,52 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K73" s="1" t="n">
-        <v>46121.54375</v>
+        <v>46122.26506944445</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>High Level City UK Ireland</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Fury at latest park stabbing horror in Sadiq's lawless London – 'where are the police?' - Daily Express</t>
+          <t>Firenze antifascista, la manifestazione a Rifredi - La Nazione</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Fury at latest park stabbing horror in Sadiq's lawless London – 'where are the police?' - Daily Express</t>
+          <t>Anti-fascist Florence, the demonstration in Rifredi - La Nazione</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 15:15:00 GMT</t>
+          <t>Thu, 09 Apr 2026 17:49:18 GMT</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxOaHVuSDctTWlmaDZQNGFFNkxEbTZ0WDk2ZHFERGpvQ1ZnV2trZHBiZUw4RnhpU3MxbTZWaFM5QVQ3anJZbXQ5VkZlME5vOTZwUWxQYnVTSnlEak9UQ2xPU2VJUWxDeXBpOUtjaEVjVFdGUmNzMzVIc2lsOXZVM2tiUTVDZEhucE1rcDdGZGFzaFJCWFh2akZ30gGcAUFVX3lxTE01M3JMS1FBUlhKM3h0aEY3enhkaFA5cy1JT0NLLW1maW1fNDh5UWpYQm9aTm5TakdUOHBsMlVWTVgyUVBhWkdCNEhBMy1QczJnZGlVaV9ITHlFSnNlZ3FaTHY5ZnprdWtQLUhmTXJra1F5NHo5ellpNmlaM2UtZUk5ektTbnFhNGVuMjd1QlB1QlRoaUF3SzJnN0F0WQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxPZlplekdZZWY3alY3TlF6SC1WZUpwY2IyWGUtd3NfSkV4RW1icW51MnFfOVRic0lHLVprY1ZYUUp2SWtBakFlZTdVYXU5MlFSWU05aWZmZ2FqZ01iQVJ3Wng0NG1NYnNaWnBMWlJ0LXVacFlTMzJHdHlXSnZmWGRfbFlsbzRCbUwtNldXblppM2c3QQ?oc=5</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -4475,52 +4475,52 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K74" s="1" t="n">
-        <v>46121.63541666666</v>
+        <v>46121.74256944445</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>High Level City UK Ireland</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>April 9: Finbar Sullivan Stabbing Spurs London Safety, Surveillance Focus - Meyka</t>
+          <t>Sciopero dei giornalisti di La7: il comunicato sindacale - TGLA7</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>April 9: Finbar Sullivan Stabbing Spurs London Safety, Surveillance Focus - Meyka</t>
+          <t>La7 journalists' strike: the union statement - TGLA7</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 22:27:16 GMT</t>
+          <t>Thu, 09 Apr 2026 20:25:00 GMT</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxPbTVXdXJwSHJybW1xWnBwd0tzTmdMMTRqamllMGlZSExhRlB2bHUtQ0Q3OHp3R3VidU9jY2ZiTllUS0FpY1gxbEFMTWhjenNuTnhveEwxMWNnd2Zray1EMm9lN2tOYzVxeG1vaE1ZTW5najdIYVp5elhzdXVXMVRRbnp0Y1F5X3kzMVVveVBXcVZjcWtwcVkyQnpuNFNjUHpaaXc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQcFdINXNScjktc05laUFkdWlpaFcySGI4cDZQbXY1S1MtM3VONHlPdHZWOU5zemtmSnZxa2JFOHdEN2t2ZlBYQk9JNzlHVHdwN1owc2FTSjdhM3B5MWFyNFBjUFM0R2prVmF1YTRXU0V6bEp1RVY0NFMwYmxXUkx5UzU1UFlYMmRuTjVBSTFZX3R3T0HSAZgBQVVfeXFMT1ZNNVhkYXhYb1dOQjhZVHRNQ0VWYVlrRWFYcWRQTW1hZTVIcGs3eExVOFdPS2Vmb2U0OHI0YUpuVExMNkZEV0NPSmZmYkh2cm5DeEpYUlROaTY2NHBEMHlON3VVVGw0WlZoMGpFbXoyMjBjdUZjUDBDbDNlQ3NQb0FMNXR6N1VnMElMclhGOTVfRUpYR0RPeVc?oc=5</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -4530,52 +4530,52 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K75" s="1" t="n">
-        <v>46121.93560185185</v>
+        <v>46121.85069444445</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>High Level City UK Ireland</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>CCTV released of men wanted in connection to shooting in London - London Now</t>
+          <t>Domani sciopero 4 ore controllori volo - RaiNews</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>CCTV released of men wanted in connection to shooting in London - London Now</t>
+          <t>Flight controllers on strike for 4 hours tomorrow - RaiNews</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 10:04:19 GMT</t>
+          <t>Thu, 09 Apr 2026 16:40:21 GMT</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQWWdyMzA2NTY5SEZtOXBWOXQ3N0xFSlpVY2xfSk1xaWRELS0tQ3E3S3Eyd0w3Rk1NLXIweUpKQ0FEN3hKQ2ROUFFtNVJQT2R5bU5YRHVLMGtMREZ2Zi0tWlgtY3RDX2RHWXVzcnBsOTRKRWxqVVRrODlwWkRwQnF1czFoWUtRRlpaLXl0UDlCUkxFMUFXV1R2c3FadDBRYjA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxNM0JodVJxV1FsNHZhRmNzRWpXM2M1SkNPYmpFUm9xVUNnTU5uaG5TcE9ZYmw5UVo3ZThIQkl3aVRZdlBDZzFrMTFkQTZER0E5bld5SFZ0ZzY3WFRBYTR0bFpSSjUyVGJwc3R6ZWVaR2xURFdGYk9Pbks5akVkRjh0a2dpeFI2SUFuWFEwVmNuUmxOeWwtc0dIMlYxbXprc3RoUmdDcldzaGlSNGNOY3JTeEZNX010NkpzLXFObFNndTRIRUhK0gHEAUFVX3lxTE0zQmh1UnFXUWw0dmFGY3NFalczYzVKQ09iakVSb3FVQ2dNTm5oblNwT1libDlRWjdlOEhCSXdpVFl2UENnMWsxMWRBNkRHQTluV3lIVnRnNjdYVEFhNHRsWlJKNTJUYnBzdHplZVpHbFREV0ZiT09uSzlqRWRGOHRrZ2l4UjZJQW5YUTBWY25SbE55bC1zR0gyVjFtemtzdGhSZ0NyV3NoaVI0Y05jclN4Rk1fTXQ2SnMtcU5sU2d1NEhFSEo?oc=5</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -4585,52 +4585,52 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K76" s="1" t="n">
-        <v>46121.41966435185</v>
+        <v>46121.6946875</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>High Level City UK Ireland</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>What we know so far as blood stains left outside café after man stabbed to death - London Now</t>
+          <t>Remigration Summit, Sala rassegnato: “Evento inappropriato, evoca deportazioni. Ma non si può evitare” - Il Giorno</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>What we know so far as blood stains left outside café after man stabbed to death - London Now</t>
+          <t>Remigration Summit, Sala resigned: "Inappropriate event, it evokes deportations. But it cannot be avoided" - Il Giorno</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 10:27:26 GMT</t>
+          <t>Fri, 10 Apr 2026 10:19:16 GMT</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQeWFOZFdzSUhZZ2ItVFdRLVIxU3IxX05tcElyUlgxX1VuMHJ0SjVaSllIbUV2N20zN05SekhuYU8ya2xneUJadFVLYXh1VTVGTHRGMjhVUjU0WW8zd2NxOFllR3dVQnhBblFHWlFyeUx3RVVzU0tpWVZnQ0xNbUJxWTl0eVVvbzlIVTFlWEVNb0JfcVNHRzdmWXpwT2trS20zTFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFBnR2h4dll1T0ZUWERBcXE5YUtBaXdXcHRZaUluSlhuUzZCMlFLV1loaU9ZSk5ybWQ1a05TV2h5UTZoSTNtRUd2Q2J4X3pVRlRBSUpGYXFDU19kZ1RmelR0eEFYM1FieEJyU1RnUFZkVWhWOFRVV3c?oc=5</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -4640,52 +4640,52 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K77" s="1" t="n">
-        <v>46121.43571759259</v>
+        <v>46122.43004629629</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>High Level City UK Ireland</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Bomb squad called to Tate Modern after visitors spot ‘suspicious package’ - Irish Mirror</t>
+          <t>Sciopero aereo il 10 aprile: voli a rischio per quattro ore in tutta Italia - Torino Cronaca</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Bomb squad called to Tate Modern after visitors spot ‘suspicious package’ - Irish Mirror</t>
+          <t>Air strike on April 10: flights at risk for four hours throughout Italy - Turin News</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 09:56:15 GMT</t>
+          <t>Thu, 09 Apr 2026 19:33:00 GMT</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxQODJyOVd4X1JBaXNpRHVId1FsWjVSSmdRZ3hfckV0LXI4UnVScXlPMVhoWlQ0TnptSFpZUS1lX2JFYUJEUE5RWHZyNGZoYXUwZ3BfeDM1a294V0REaUUxWWxzd2FMUVlubnhRRExaREJwLWFFQXlldFBWVTZBX3kxNnlCbDlTdHlm0gGOAUFVX3lxTE0tYURkX0hMLU1nZlVlQmRSX3hGczM5d016M0U4Nm5NSE5Ib1NlSXlFdGV5RVF3WU96UlhqNnM5Q0pCOXhYX2RUZWlXcjJrVTR5aEhXRGVLcXZuSXFKT1lCWXhpSXBCamNiVkxZVlN4M3dvVzdpLUt4TDRMWDFyWkk0eXhJUElNSkhrcVNVQmc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPOHFUUmtqeGJvcFhtanNDdXpDeFFGaEVCWEd5YkVNbHhVY0Y5Q0ZobVd4S1NZRC1uQ2JCUjI5RThsQzVvcGJxUWFFZ1FpQ3pvOXdKd2Yxa0NIdjZ1Y2pmamJxcDdvekxCb0E0V0Fqc0p3UDZEaGM0WUFoQ09wOWdWb3dOQ21iN1BxMDZMY0FncTI2SUdiaTRkb3phTDgtWWRhRlpTY2lmLVkwY1dUbHQ2TGN5QWVkMVZ5T19VeTFxYmFJSUE?oc=5</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -4695,52 +4695,52 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K78" s="1" t="n">
-        <v>46121.4140625</v>
+        <v>46121.81458333333</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>High Level City UK Ireland</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Camberwell shooting first photos as man raced to hospital with gun shot wound - My London</t>
+          <t>Hannoun manifestazione milano duomo - Contropiano</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Camberwell shooting first photos as man raced to hospital with gun shot wound - My London</t>
+          <t>Hannoun event Milan Cathedral - Contropiano</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 14:52:14 GMT</t>
+          <t>Thu, 09 Apr 2026 12:45:02 GMT</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQSXJYcm1IX01kSk5ZOHd3cTRHczF0ajlGd2NTQTdoX3p1SVZwU2htRzlhZXdwU1NadHpJUGJOZW1YWDQ2VmR0N2lzeV9Xb0hIaTBWMXIyV0Y5VjVtUS1SdlBOcTE2WlBwUkc3dFE1RWc5blI4Qnc3TGwwY3BEUlV4SGF2SzlMM3dmNjRQMXVDeWhsZ0d5aXU5cUFZUXBPeWhsVERPY9IBqgFBVV95cUxPQlNSVXF2WEx5UlktSFRsUnRSNFRySWVYMG5oTEl2cm5KREdaWWpGUnBhelBwME1kOGYzZzJhNVNHNHN0dE8yZFZzdWhta1l4SFg0aDhnUVFUQjFRQ1ZROHU2Wk1Qc2MzQkVlZHBwc2pIQy1JWTBGUG8wOVBpWkt3OTF1NkZRanN6cmg4T1huZEhmU0x3TE8xT2s1MXFQRnQ4a0hlOUlFcW9Mdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgJBVV95cUxNNDBVLXBuQzhaS0VCTUxGaTB1dXBTTE1lVXBJWkZKRWdwaUNIWDBQSnZVQ0VSUWhYUDh5bWZJTXdKLWhvZ3ctYnBnaEl2Q1FuM3FJelNnM0Y5NTZJNEtOV29rM2tTSEhod1hVcG9HVDdHX3RXWHpJNmk4UTRKLVdnal8zTllWRlpNRkpQU2xIOUZiZkJLa3ptYjRNd3hFYzEwaTE4dmcxaFNMMmNpTzFXNHpxNmRyeEJfbnZwakkwelpvYmIyRXFzODc3Tnd1Vm5LeXgzdDk2LWt2YWpDVS1kdFZtaGxXcWFjRHo2eDNXazFZVS1zN1dJNHJfYmdvcS05U191Y21xSkpaZXo4Z0N1enh5R1VfaXRMbjVPd1NlRXM5dTZUczFLVk1n?oc=5</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -4750,52 +4750,52 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K79" s="1" t="n">
-        <v>46121.61960648148</v>
+        <v>46121.53127314815</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Village La Vallee (fallback)</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>("La Vallee Village" OR "La Vallée Village" OR "Serris" OR "Chessy") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>United to win: Scouts in Paris hold charity Easter egg workshops and raise over 800 euros for Ukraine’s armed forces - Рубрика</t>
+          <t>Trasloco della caserma: "Ma resti un presidio" - Il Giorno</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>United to win: Scouts in Paris hold charity Easter egg workshops and raise over 800 euros for Ukraine’s armed forces - Рубрика</t>
+          <t>Moving of the barracks: "But it remains a garrison" - Il Giorno</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 14:57:41 GMT</t>
+          <t>Fri, 10 Apr 2026 04:33:11 GMT</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE5wRWpBT2d1SGxYcGJNaldGOXpuMnN4RXp2MXRfa0hRelhUY01SMEJXYzVOZHVNUDhqeGJjeE1KTWl4SXFwRHJ1bG14R3NZNXhWUGN3UUplWVFFemJFSFMwaTdzRW5LcGNSQWVvcmpOV3k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxPb1kzWmY4RENXeEVHaE5BaTFfcUZubGw2X3dMTXI1NnZMTEtYLUViaEgtektQYzlyMlJIejJMc1lDdWhnSkVIVnA2YXVVUkwtRnpIVlFJZzdqaDZPUWVGNnR2UkR5QUpub3VKWDJKam1zaTVlUzdPdl9fazYyZUZVdWhvaTlWdw?oc=5</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -4805,52 +4805,52 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K80" s="1" t="n">
-        <v>46121.62339120371</v>
+        <v>46122.18971064815</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>High Level City Italy English</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>("Milan" OR "Milano" OR "Bologna") AND ("Italy" OR "Italian") AND (protest OR demonstration OR rally OR "civil unrest" OR strike OR blockade OR march) AND -football AND -transfer AND -Serie AND -"fashion week" AND -catwalk AND -runway</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Italian Air Traffic Controllers Set for 4-Hour National Strike on 10 April—Hundreds of Flights Already Cancelled - VisaHQ</t>
+          <t>Scioperi a raffica da domani: trasporti a rischio per tutto aprile - La Nuova Provincia</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Italian Air Traffic Controllers Set for 4-Hour National Strike on 10 April—Hundreds of Flights Already Cancelled - VisaHQ</t>
+          <t>Rapid strikes starting tomorrow: transport at risk for the whole of April - La Nuova Provincia</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 22:09:14 GMT</t>
+          <t>Thu, 09 Apr 2026 13:00:47 GMT</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxNTEZyb0gwVjI0V1FaTjg4VXluWV82aWJfa1dLUk1UdmE1b0xDR1J5ZTNmdzFyaENQMm1Lc3dCSWVEbnhIYi1NdHMwQldYbGhPQ1dpNnBtOTdRX1U3N2RlM1F6dkNCUWdYVWQzeTRnV1hxS191OHkwUjBuTzFRa0w0ZDNXb29NTzZva3hVcTh1WHVDSWNvQ3VkYUo1S1BqY0xLcURULWszd3hpbEtET2VlRTBZQjV6M01xY1F2dkdQOTY3eHdaT0tUSENJSW1ISTFwWmdmeG9EMzZlRnEzOEQ0b29ZZ0MzRTFQZEVR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQdHd3ek9ybDQ5MGNZSHkycnp5VjBLemZKM2szNTNpUENBSXVEY0ZDQ1BJcmNVSUpWWU1oWGt1Zmt5QjdsMUpWbmZ0eWxLc1dWY09yMGJBcnhlR1hfVWp4SVQ5em1acllNMG1QX0NMbFdnSDRnem9ON21yYXhmVzZ2X0RNLTZ6VDJQT0M2Y25ZLTRTdXRaVmtCSTdDeWs5RldGbzRPcHNZMmkyd2R5QmhNZUg5Q1FRdw?oc=5</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -4860,7 +4860,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -4870,42 +4870,42 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>IT:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K81" s="1" t="n">
-        <v>46121.9230787037</v>
+        <v>46121.54221064815</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>High Level City Italy English</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>("Milan" OR "Milano" OR "Bologna") AND ("Italy" OR "Italian") AND (protest OR demonstration OR rally OR "civil unrest" OR strike OR blockade OR march) AND -football AND -transfer AND -Serie AND -"fashion week" AND -catwalk AND -runway</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>FTSE MIB Today: Milan Edges Lower as Italy's Blue-Chips Consolidate Ceasefire Rally - BBN Times</t>
+          <t>Remigration Summit, alta tensione: due contromanifestazioni Antifa, polemica in Comune e Regione - Il Giorno</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>FTSE MIB Today: Milan Edges Lower as Italy's Blue-Chips Consolidate Ceasefire Rally - BBN Times</t>
+          <t>Remigration Summit, high tension: two Antifa counter-demonstrations, controversy in the Municipality and Region - Il Giorno</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 20:04:23 GMT</t>
+          <t>Fri, 10 Apr 2026 00:45:52 GMT</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxNM0V0TzBvQm9SWlFTV1VONldxVjN0bzRqYjlIRzZRRDlzeEQ3OVdTTWt5c3AwVE4yUVQ3T1ZfeFB4UUhqbHpuc0lTRDlodW01MHVSZEFhN1dlZHJJaGNYRmg3eWdza1FjLTc5M0xQV21YMVpEOFBwU3pKMVdnb3pNeWFoRmhjLWlwQndiRWw0aEtIZUIzRXJ1OFBQUTFMMV85OUM0c1pwUkd0U2RTTjJfR3RkamlFV3JYdkNRb0xBSlFLTi05WkJMNy01djB6Zw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE9Pc3JOX3I5MnM2SjhVOFFBOFJUekpINUdUcDBGdTBOS09hRU50Z1dIQmlXN1lyS0FQQkExVmNQRXhKQmtVMXF2TUFGUDBickFJZzVXQmFMWHU4YkJOemNKOUVfRmFObGZFekY2Ui1BWkFQbWYwZ0E?oc=5</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -4915,7 +4915,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -4925,11 +4925,11 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>IT:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K82" s="1" t="n">
-        <v>46121.83637731482</v>
+        <v>46122.03185185185</v>
       </c>
     </row>
     <row r="83">
@@ -4945,22 +4945,22 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Sanità pubblica, sabato 11 aprile a Milano la manifestazione regionale davanti a Palazzo Lombardia - FP CGIL Lombardia</t>
+          <t>Sciopero aereo anche a Malpensa e Linate: Ita elimina il 27% dei voli - Mi-Tomorrow</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Public health, the regional demonstration in Milan on Saturday 11 April in front of Palazzo Lombardia - FP CGIL Lombardia</t>
+          <t>Air strike also at Malpensa and Linate: ITA eliminates 27% of flights - Mi-Tomorrow</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 10:02:22 GMT</t>
+          <t>Fri, 10 Apr 2026 07:22:01 GMT</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxQUFZLbWgwTDhMRGZaTFB2eHRSaTVJQks0eFcxQTY2dEluX0xtWkN5a3JRcm5TSHA5dm84VHdHV0VjSTYwODktc0hHMWhvWlhuNTBoLTVKUkliNEhrd0VXQXkzQk1lM2YzZXdLUjBFdVNKQThDNlBXa3o1Z0ZwZVF1M0k0WDVIeC1nU0pJZlo3OXdBVWR5WjZfeUlwbHF1UQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE5QT1hXUUJPb3Q4UW9uRWNoYjdXbXBWb24tTjNlemRMOXg2empTYUh4THRueHFiaUZDNC14aTRnOW54TFBMcmpYLUQ2OHJfMWVtUGFaUWRVNFVuakhmRFhTWGZFdWZqV0RiQ2JFMUdjQmJSR0V2Qk0teWFR?oc=5</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -4984,7 +4984,7 @@
         </is>
       </c>
       <c r="K83" s="1" t="n">
-        <v>46121.41831018519</v>
+        <v>46122.30695601852</v>
       </c>
     </row>
     <row r="84">
@@ -5000,22 +5000,22 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>MILANO: “FERMIAMO IL TERRORE SIONISTA, CONTRO L’AGGRESSIONE GENOCIDA SUL LIBANO” PRESIDIO IN PIAZZA DELLA SCALA - Radio Onda d`Urto</t>
+          <t>Sanità, sabato 11 aprile la protesta sotto il Pirellone: "La salute è un diritto, non una merce" - Varese7Press</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>MILAN: “LET'S STOP THE ZIONIST TERROR, AGAINST THE GENOCIDAL AGGRESSION ON LEBANON” PRESIDENT IN PIAZZA DELLA SCALA - Radio Onda d`Urto</t>
+          <t>Healthcare, protest under the Pirellone on Saturday 11 April: "Health is a right, not a commodity" - Varese7Press</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Thu, 09 Apr 2026 11:35:00 GMT</t>
+          <t>Thu, 09 Apr 2026 11:52:37 GMT</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxNVllxY2RBYTNudTVwMkk4TFR1TXgwbV9USmpybmNXUERuMU1veGVZUzRxSlNvejc0MDVjQ3p2dmJ4amxEbE5qVXA5VkZGN2VMd2xjSTVXMlZEa29XN2wxQVBCcFRoT1Z5OFYzdDhhZ0pzMUlHa2N6NGxlaFpRdHVacmJNWkkxVTJSZVNEUVlqT1ltUWFYOHJ0ZE4xNE15Vm85Q05MV3pJU1JuLXlEblRybnowNjhwWkpWRlNRbjkxck5uYWJrb1d6MGhUZVFDWHpSbE1QQUNNTnVqNWptUHVoQzNR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxNeWJpblRjRXZYQUdIaWU5TGl4SU9VYTlpSVl3UmsxNzBtUXktRXQ4bnFBRFZ1QVdwd2YtSkNWYmxxODgwVUFvNDRuMXBvNGtLcGZfYWc1aE8wZW5SSVpDdHQ4ZkVIS2plTFN1ZS02YjRPMmhMQlFjS2htRXRQY3FONl9TQlBlazkxTUlaazdBM3E4OFVOMTJwaE1xdU04WHNaU2o3cGNWd2VRNHFkQnRQLW9lZGxrVmstUXJSSjhONVlXT2RyT2xDYVh1VdIB0AFBVV95cUxNQ1pPSjJtNXFYZWdaYng5dHk3c0V1VE1xNDBuTDRuM3RGc1NYTmJ5MG5IaTZHRklqVHFIbHBHZzBOODVDZlB1Y2t3OF9wRTZyTXgzWk8zLWsxWmJfUzVjblVILXJDMHlLVFRzUEJKMVJmaXY5X3hWSWFGeWFXU1JjMEN4WnNkQjdUWmVzZ00zWnFQZHR0cWhjdGZCYTlmQklLTldqdEpsS2I4Uk9acndhWFE2cVZCMDRyUTZOekZGMDhCenY1cFE0QUtEbENadXNO?oc=5</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -5039,942 +5039,7 @@
         </is>
       </c>
       <c r="K84" s="1" t="n">
-        <v>46121.48263888889</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>Consorzio Cineca, sciopero e doppia manifestazione a Roma e Bologna il 10 aprile - Filcams Cgil</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>Cineca Consortium, strike and double demonstration in Rome and Bologna on 10 April - Filcams Cgil</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>Thu, 09 Apr 2026 09:37:36 GMT</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxPclJ6Q1g0STBrV25QVWFiZFJXSkhPQkV6REo1QXlXb0M4WktpTHI5OENISjkwZWk3Sm9jMzdoelp6bU82bXF4bkk5QVFFRjZPS0J2WkdpWXh6a1E4aVBYb1BVd3dPY2hNQ2J0S2dwQW5YYkRWN3hHZ3VQYWQydjYxM25Pd3hValNtblZrQlpUbG10THRnZ1I3ZjZwVUpnODZZV1pZQ2FpUlY0cnpHV2tyam1xS1daUnoxb2Rnc185WS1NLTB6b1lj0gHHAUFVX3lxTE9yUnpDWDRJMGtXblBVYWJkUldKSE9CRXpESjVBeVdvQzhaS2lMcjk4Q0hKOTBlaTdKb2MzN2h6WnptTzZtcXhuSTlBUUVGNk9LQnZaR2lZeHprUThpUFhvUFV3d09jaE1DYnRLZ3BBblhiRFY3eEdndVBhZDJ2NjEzbk93eFVqU21uVmtCWlRsbXRMdGdnUjdmNnBVSmc4NllXWllDYWlSVjRyekdXa3JqbXFLV1pSejFvZGdzXzlZLU0tMHpvWWM?oc=5</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H85" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J85" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K85" s="1" t="n">
-        <v>46121.40111111111</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>Firenze antifascista, la manifestazione a Rifredi - La Nazione</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>Anti-fascist Florence, the demonstration in Rifredi - La Nazione</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>Thu, 09 Apr 2026 17:48:47 GMT</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxPZlplekdZZWY3alY3TlF6SC1WZUpwY2IyWGUtd3NfSkV4RW1icW51MnFfOVRic0lHLVprY1ZYUUp2SWtBakFlZTdVYXU5MlFSWU05aWZmZ2FqZ01iQVJ3Wng0NG1NYnNaWnBMWlJ0LXVacFlTMzJHdHlXSnZmWGRfbFlsbzRCbUwtNldXblppM2c3QQ?oc=5</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J86" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K86" s="1" t="n">
-        <v>46121.74221064815</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>Sciopero aerei 10 aprile 2026: stop Ita Airways, Ryanair, Easyjet - BusinessMobility.travel</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>Sciopero aerei 10 aprile 2026: stop Ita Airways, Ryanair, Easyjet - BusinessMobility.travel</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>Fri, 10 Apr 2026 01:17:42 GMT</t>
-        </is>
-      </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQakM4UEVUdURxZXNIYWlmNE5mUWtTM1FDdWxiSU41WEx3MVRMc1ZmX2FPUWk5SnRBa09LZEhyXzc1a2ZUd01FQ3BpMzNkcUo3UERrUnJTT3J0T1pCblhacDYxV204SDNLWERfdVlubHFVOUVPdFlKVFVyekhOdThhM2hBVnB4ck9nRTZ4Q3owRGtyd2wwTF9nUnRRNVFXOFpkcDVhdEhNYnU?oc=5</t>
-        </is>
-      </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H87" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J87" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K87" s="1" t="n">
-        <v>46122.05395833333</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>Scintille sul Remigration Summit del 18 aprile, Forza Italia: iniziativa razzista. Pd: facciano cadere governo allora - Il Giorno</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>Sparks on the Remigration Summit on April 18, Forza Italia: racist initiative. Pd: let the government fall then - Il Giorno</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>Thu, 09 Apr 2026 17:18:43 GMT</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxNd09BUkxPUTMzT2VNdEU2VVIwb0I3blo4YVpRLWY2cHJBbjVJUk12OFRkTmVCTWNNTUtTMXdSd05YeGU4cTV0Uy0yNWJVdXZxdWc1eDJtcmN2R21VbWhwMUlER2dmNkFJeEJXeEl1WmUzN0N0V1hFMm5LQkNMVmNkWmM5OA?oc=5</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H88" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J88" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K88" s="1" t="n">
-        <v>46121.72133101852</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>Milano: Lega protesta contro no a Remigration summit, ”stop Fascismo rosso” - Foto - Agenzia Nova</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>Milan: Lega protests against no to Remigration summit, "stop red Fascism" - Photo - Agenzia Nova</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>Thu, 09 Apr 2026 21:19:53 GMT</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxNd0EyWjRKMnlkRWVjSkxzZ1VUUVk5dXNHelF1VzB1dVZ0REhJVHlUQXVVZndlQ3d0VWpJRUVvQ0FFTmw2WE5qRldERU96ZzdxZ1hjWTR2dFFHeXhNaTVDQXNRQmxydnFmd3ZHOTBUZXJuOW5qZlpnOW9Fcm9lS19KdlZ2MmlWWXpQemNUV1RZTE5CRC1taFlpejV6M0E1XzdrRlYwRkY3cXNxY3Q0dWJhN1FTWTZpNGVqRENRVkh0eU13NGtrdWJFR2ZiSThDSjB3VXlkd0FYdE90dFNxZGM0S2tpZw?oc=5</t>
-        </is>
-      </c>
-      <c r="G89" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H89" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I89" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J89" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K89" s="1" t="n">
-        <v>46121.88880787037</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>Hannoun manifestazione milano duomo - Contropiano</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>Hannoun event Milan Cathedral - Contropiano</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>Thu, 09 Apr 2026 12:45:02 GMT</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiqgJBVV95cUxNNDBVLXBuQzhaS0VCTUxGaTB1dXBTTE1lVXBJWkZKRWdwaUNIWDBQSnZVQ0VSUWhYUDh5bWZJTXdKLWhvZ3ctYnBnaEl2Q1FuM3FJelNnM0Y5NTZJNEtOV29rM2tTSEhod1hVcG9HVDdHX3RXWHpJNmk4UTRKLVdnal8zTllWRlpNRkpQU2xIOUZiZkJLa3ptYjRNd3hFYzEwaTE4dmcxaFNMMmNpTzFXNHpxNmRyeEJfbnZwakkwelpvYmIyRXFzODc3Tnd1Vm5LeXgzdDk2LWt2YWpDVS1kdFZtaGxXcWFjRHo2eDNXazFZVS1zN1dJNHJfYmdvcS05U191Y21xSkpaZXo4Z0N1enh5R1VfaXRMbjVPd1NlRXM5dTZUczFLVk1n?oc=5</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H90" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J90" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K90" s="1" t="n">
-        <v>46121.53127314815</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>Sciopero trasporti 10 aprile: chi rischia di restare a piedi e le fasce orarie da bollino rosso per aerei e bus - Studenti.it</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>Transport strike 10 April: those who risk being left on foot and the red flag time slots for planes and buses - Studenti.it</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>Thu, 09 Apr 2026 10:12:00 GMT</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPdzBzRmRiMDB4b0JPRTROV3FFZTZwNzJwckNhV3ZzSmFtUHI0Q2ppOEhGT2pBaU1iT0x4TEFBMEJTQVBDVWxTa1NDS2gzeE1Sa3p2R3Z3ZmFGN1NRM3BscGtuVmFLSUdIeEFiaV9FbWNMcDRwNWJxYjYxUmRHcjFZNUdTZUZYdi11SnJzeDkzNXk1UWV3aG0wdktWa1ZlM0pqZHdFb1h6ZllXekl4cHJBVV9qcmZYcHh4a0VfSjV5VV9GZzcyWExBTUZZN1pIY1Vxa2l1OTFB?oc=5</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J91" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K91" s="1" t="n">
-        <v>46121.425</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>Domani sciopero 4 ore controllori volo - RaiNews</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>Flight controllers on strike for 4 hours tomorrow - RaiNews</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>Thu, 09 Apr 2026 16:40:21 GMT</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxNM0JodVJxV1FsNHZhRmNzRWpXM2M1SkNPYmpFUm9xVUNnTU5uaG5TcE9ZYmw5UVo3ZThIQkl3aVRZdlBDZzFrMTFkQTZER0E5bld5SFZ0ZzY3WFRBYTR0bFpSSjUyVGJwc3R6ZWVaR2xURFdGYk9Pbks5akVkRjh0a2dpeFI2SUFuWFEwVmNuUmxOeWwtc0dIMlYxbXprc3RoUmdDcldzaGlSNGNOY3JTeEZNX010NkpzLXFObFNndTRIRUhK0gHEAUFVX3lxTE0zQmh1UnFXUWw0dmFGY3NFalczYzVKQ09iakVSb3FVQ2dNTm5oblNwT1libDlRWjdlOEhCSXdpVFl2UENnMWsxMWRBNkRHQTluV3lIVnRnNjdYVEFhNHRsWlJKNTJUYnBzdHplZVpHbFREV0ZiT09uSzlqRWRGOHRrZ2l4UjZJQW5YUTBWY25SbE55bC1zR0gyVjFtemtzdGhSZ0NyV3NoaVI0Y05jclN4Rk1fTXQ2SnMtcU5sU2d1NEhFSEo?oc=5</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H92" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J92" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K92" s="1" t="n">
-        <v>46121.6946875</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>Sciopero dei giornalisti di La7: il comunicato sindacale - TGLA7</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>La7 journalists' strike: the union statement - TGLA7</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>Thu, 09 Apr 2026 20:25:00 GMT</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQcFdINXNScjktc05laUFkdWlpaFcySGI4cDZQbXY1S1MtM3VONHlPdHZWOU5zemtmSnZxa2JFOHdEN2t2ZlBYQk9JNzlHVHdwN1owc2FTSjdhM3B5MWFyNFBjUFM0R2prVmF1YTRXU0V6bEp1RVY0NFMwYmxXUkx5UzU1UFlYMmRuTjVBSTFZX3R3T0HSAZgBQVVfeXFMT1ZNNVhkYXhYb1dOQjhZVHRNQ0VWYVlrRWFYcWRQTW1hZTVIcGs3eExVOFdPS2Vmb2U0OHI0YUpuVExMNkZEV0NPSmZmYkh2cm5DeEpYUlROaTY2NHBEMHlON3VVVGw0WlZoMGpFbXoyMjBjdUZjUDBDbDNlQ3NQb0FMNXR6N1VnMElMclhGOTVfRUpYR0RPeVc?oc=5</t>
-        </is>
-      </c>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H93" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I93" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J93" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K93" s="1" t="n">
-        <v>46121.85069444445</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>Sciopero aereo il 10 aprile: voli a rischio per quattro ore in tutta Italia - Torino Cronaca</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>Air strike on April 10: flights at risk for four hours throughout Italy - Turin News</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>Thu, 09 Apr 2026 19:33:00 GMT</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPOHFUUmtqeGJvcFhtanNDdXpDeFFGaEVCWEd5YkVNbHhVY0Y5Q0ZobVd4S1NZRC1uQ2JCUjI5RThsQzVvcGJxUWFFZ1FpQ3pvOXdKd2Yxa0NIdjZ1Y2pmamJxcDdvekxCb0E0V0Fqc0p3UDZEaGM0WUFoQ09wOWdWb3dOQ21iN1BxMDZMY0FncTI2SUdiaTRkb3phTDgtWWRhRlpTY2lmLVkwY1dUbHQ2TGN5QWVkMVZ5T19VeTFxYmFJSUE?oc=5</t>
-        </is>
-      </c>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H94" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I94" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J94" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K94" s="1" t="n">
-        <v>46121.81458333333</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>Nuovo sciopero dei treni l'11 aprile: viaggi a rischio nel week end - NovaraToday</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>New train strike on April 11th: travel at risk over the weekend - NovaraToday</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>Thu, 09 Apr 2026 12:54:47 GMT</t>
-        </is>
-      </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE95NXFTMks5ODJoSjNsMlZqZW1vVl85dllZRW1NYTlvRDVMYnJsWU1NUklQV3ZPMXp3XzUwT19OMHR5NUxXRnd2UTlqUHJhc3I0QndWZ3E2MmxYNXlON3BaZFJpaTZRWU5Wbm1hWHFwYjFjNjBzRDViNnhIMA?oc=5</t>
-        </is>
-      </c>
-      <c r="G95" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H95" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I95" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J95" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K95" s="1" t="n">
-        <v>46121.53804398148</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>Scioperi a raffica da domani: trasporti a rischio per tutto aprile - La Nuova Provincia</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>Rapid strikes starting tomorrow: transport at risk for the whole of April - La Nuova Provincia</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>Thu, 09 Apr 2026 13:00:47 GMT</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQdHd3ek9ybDQ5MGNZSHkycnp5VjBLemZKM2szNTNpUENBSXVEY0ZDQ1BJcmNVSUpWWU1oWGt1Zmt5QjdsMUpWbmZ0eWxLc1dWY09yMGJBcnhlR1hfVWp4SVQ5em1acllNMG1QX0NMbFdnSDRnem9ON21yYXhmVzZ2X0RNLTZ6VDJQT0M2Y25ZLTRTdXRaVmtCSTdDeWs5RldGbzRPcHNZMmkyd2R5QmhNZUg5Q1FRdw?oc=5</t>
-        </is>
-      </c>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H96" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I96" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J96" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K96" s="1" t="n">
-        <v>46121.54221064815</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>Trasloco della caserma: "Ma resti un presidio" - Il Giorno</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>Moving of the barracks: "But it remains a garrison" - Il Giorno</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>Fri, 10 Apr 2026 04:33:11 GMT</t>
-        </is>
-      </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxPb1kzWmY4RENXeEVHaE5BaTFfcUZubGw2X3dMTXI1NnZMTEtYLUViaEgtektQYzlyMlJIejJMc1lDdWhnSkVIVnA2YXVVUkwtRnpIVlFJZzdqaDZPUWVGNnR2UkR5QUpub3VKWDJKam1zaTVlUzdPdl9fazYyZUZVdWhvaTlWdw?oc=5</t>
-        </is>
-      </c>
-      <c r="G97" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H97" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I97" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J97" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K97" s="1" t="n">
-        <v>46122.18971064815</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>Remigration Summit, alta tensione: due contromanifestazioni Antifa, polemica in Comune e Regione - Il Giorno</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>Remigration Summit, high tension: two Antifa counter-demonstrations, controversy in the Municipality and Region - Il Giorno</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>Fri, 10 Apr 2026 00:45:52 GMT</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE9Pc3JOX3I5MnM2SjhVOFFBOFJUekpINUdUcDBGdTBOS09hRU50Z1dIQmlXN1lyS0FQQkExVmNQRXhKQmtVMXF2TUFGUDBickFJZzVXQmFMWHU4YkJOemNKOUVfRmFObGZFekY2Ui1BWkFQbWYwZ0E?oc=5</t>
-        </is>
-      </c>
-      <c r="G98" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H98" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I98" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J98" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K98" s="1" t="n">
-        <v>46122.03185185185</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>Sanità, sabato 11 aprile la protesta sotto il Pirellone: "La salute è un diritto, non una merce" - Varese7Press</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>Healthcare, protest under the Pirellone on Saturday 11 April: "Health is a right, not a commodity" - Varese7Press</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>Thu, 09 Apr 2026 11:52:37 GMT</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxNeWJpblRjRXZYQUdIaWU5TGl4SU9VYTlpSVl3UmsxNzBtUXktRXQ4bnFBRFZ1QVdwd2YtSkNWYmxxODgwVUFvNDRuMXBvNGtLcGZfYWc1aE8wZW5SSVpDdHQ4ZkVIS2plTFN1ZS02YjRPMmhMQlFjS2htRXRQY3FONl9TQlBlazkxTUlaazdBM3E4OFVOMTJwaE1xdU04WHNaU2o3cGNWd2VRNHFkQnRQLW9lZGxrVmstUXJSSjhONVlXT2RyT2xDYVh1VdIB0AFBVV95cUxNQ1pPSjJtNXFYZWdaYng5dHk3c0V1VE1xNDBuTDRuM3RGc1NYTmJ5MG5IaTZHRklqVHFIbHBHZzBOODVDZlB1Y2t3OF9wRTZyTXgzWk8zLWsxWmJfUzVjblVILXJDMHlLVFRzUEJKMVJmaXY5X3hWSWFGeWFXU1JjMEN4WnNkQjdUWmVzZ00zWnFQZHR0cWhjdGZCYTlmQklLTldqdEpsS2I4Uk9acndhWFE2cVZCMDRyUTZOekZGMDhCenY1cFE0QUtEbENadXNO?oc=5</t>
-        </is>
-      </c>
-      <c r="G99" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H99" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I99" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J99" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K99" s="1" t="n">
         <v>46121.49487268519</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>Il Pd vuole bloccare la piazza di Salvini. "Non è democratica" - il Giornale</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>The Democratic Party wants to block Salvini's square. "It's not democratic" - il Giornale</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>Thu, 09 Apr 2026 10:04:14 GMT</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPTlFnNlFQellSQXQ1U3lWRTU0Rmw2TXpZZFNudFYxMnh6UVhaZkVHalRtWXRiX2VaY1pha2tXaXA1dV9rdU4wODF1X1FLX0RQb2FIWWE2TVZ5NkMxZmpXbTZocktmU2xCOGFhYUNnVG8xOXQ3aTgwcUVKdVpIY3EwNFJ5RUhzOVFpTVFveXFaY0gyQmNwSHppYjRQbWZ5LWdaZ1hN?oc=5</t>
-        </is>
-      </c>
-      <c r="G100" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H100" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I100" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J100" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K100" s="1" t="n">
-        <v>46121.41960648148</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>Venerdì nero dei cieli, ore di sciopero, un'intera giornata di caos: l'elenco dei voli garantiti - La Sicilia</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>Black Friday of the skies, hours of strike, a whole day of chaos: the list of guaranteed flights - Sicily</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>Thu, 09 Apr 2026 17:51:32 GMT</t>
-        </is>
-      </c>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQcFg0T3BsZ1VPdEhSWmRWbnN0ZHlwMnpybjl0Q0wzSU1hRTFPR3ktWjQ4U0J2SzM3ZHpxV0hQanlZRG1VNHlNZGdDREtsUTBMeUFnOG5NOFJaNnJiWldpR2I0VVRWdlUydHJuUGtaNG1tdzZYMnlwZXZBcUlJMVYwUDNzZ0xsSWJzakpTNjRDNVpUQWRWRFdSZ0ZjTEd2bzJDbGE3U29DRDN3OTFpbjZvNEtlUVF2VWk2NlQyajg0a3hmQ0IyeVVtUTI2cjg2dG5WWVlsMFBrN0w4RlVsV05yMkJZNA?oc=5</t>
-        </is>
-      </c>
-      <c r="G101" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H101" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I101" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J101" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K101" s="1" t="n">
-        <v>46121.74412037037</v>
       </c>
     </row>
   </sheetData>

</xml_diff>